<commit_message>
added new additional functions. Wrote user_progress.db. Still need to troubleshoot the engine code to get connected with user_progress.db
</commit_message>
<xml_diff>
--- a/data/master_sheets.xlsx
+++ b/data/master_sheets.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Content_Master" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="77">
   <si>
     <t xml:space="preserve">Georgian</t>
   </si>
@@ -232,6 +232,9 @@
   </si>
   <si>
     <t xml:space="preserve">Content_Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step_Order</t>
   </si>
   <si>
     <t xml:space="preserve">Content</t>
@@ -259,7 +262,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -320,19 +323,6 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -382,7 +372,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -409,14 +399,6 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -505,7 +487,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P33"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.23"/>
@@ -1200,7 +1182,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.5"/>
   </cols>
@@ -1328,7 +1310,7 @@
       <c r="D6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="4" t="s">
         <v>43</v>
       </c>
       <c r="G6" s="4" t="s">
@@ -1647,8 +1629,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H955"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I955"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.06"/>
@@ -1656,8 +1638,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20.76"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1676,14 +1658,17 @@
       <c r="E1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="1" t="s">
         <v>69</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="1" t="s">
         <v>71</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1691,7 +1676,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>1</v>
@@ -1703,19 +1688,22 @@
         <v>1</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="10"/>
+      <c r="I2" s="8"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>1</v>
@@ -1727,19 +1715,22 @@
         <v>1</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="10"/>
+      <c r="I3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>1</v>
@@ -1751,19 +1742,22 @@
         <v>1</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G4" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="10"/>
+      <c r="I4" s="8"/>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>1</v>
@@ -1775,19 +1769,22 @@
         <v>1</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G5" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="I5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>1</v>
@@ -1799,13 +1796,16 @@
         <v>2</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>74</v>
+      <c r="I6" s="7" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1813,7 +1813,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>1</v>
@@ -1825,19 +1825,22 @@
         <v>2</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G7" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="10"/>
+      <c r="I7" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>1</v>
@@ -1849,19 +1852,22 @@
         <v>2</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="I8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>1</v>
@@ -1873,12 +1879,15 @@
         <v>2</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="G9" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="H9" s="10"/>
+      <c r="I9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4"/>
@@ -1888,7 +1897,8 @@
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
-      <c r="H10" s="9"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4"/>
@@ -1898,7 +1908,8 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
-      <c r="H11" s="10"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4"/>
@@ -1908,7 +1919,8 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
-      <c r="H12" s="10"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4"/>
@@ -1918,7 +1930,8 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
-      <c r="H13" s="10"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4"/>
@@ -1928,7 +1941,8 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
-      <c r="H14" s="10"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4"/>
@@ -1938,7 +1952,8 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
-      <c r="H15" s="10"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4"/>
@@ -1948,7 +1963,8 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
-      <c r="H16" s="9"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4"/>
@@ -1958,7 +1974,8 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="10"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4"/>
@@ -1968,7 +1985,8 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
-      <c r="H18" s="10"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4"/>
@@ -1978,7 +1996,8 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
-      <c r="H19" s="10"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4"/>
@@ -1988,7 +2007,8 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
-      <c r="H20" s="10"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4"/>
@@ -1998,7 +2018,8 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
-      <c r="H21" s="9"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4"/>
@@ -2008,7 +2029,8 @@
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
-      <c r="H22" s="10"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4"/>
@@ -2018,7 +2040,8 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
-      <c r="H23" s="10"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="8"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4"/>
@@ -2028,7 +2051,8 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="10"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4"/>
@@ -2038,7 +2062,8 @@
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
-      <c r="H25" s="10"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="8"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4"/>
@@ -2048,7 +2073,8 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
-      <c r="H26" s="9"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4"/>
@@ -2058,7 +2084,8 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
-      <c r="H27" s="10"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="8"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4"/>
@@ -2068,7 +2095,8 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
-      <c r="H28" s="10"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="8"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4"/>
@@ -2078,7 +2106,8 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
-      <c r="H29" s="10"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="8"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4"/>
@@ -2088,7 +2117,8 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
-      <c r="H30" s="10"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="8"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4"/>
@@ -2098,7 +2128,8 @@
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
-      <c r="H31" s="10"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="8"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4"/>
@@ -2108,7 +2139,8 @@
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
-      <c r="H32" s="9"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4"/>
@@ -2118,7 +2150,8 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
-      <c r="H33" s="10"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="8"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4"/>
@@ -2128,7 +2161,8 @@
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="H34" s="10"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="8"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4"/>
@@ -2138,7 +2172,8 @@
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
-      <c r="H35" s="10"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="8"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4"/>
@@ -2148,7 +2183,8 @@
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
-      <c r="H36" s="10"/>
+      <c r="H36" s="4"/>
+      <c r="I36" s="8"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4"/>
@@ -2158,7 +2194,8 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
-      <c r="H37" s="10"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="8"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4"/>
@@ -2168,2758 +2205,2759 @@
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
-      <c r="H38" s="10"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="8"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H39" s="10"/>
+      <c r="I39" s="8"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H40" s="10"/>
+      <c r="I40" s="8"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H41" s="10"/>
+      <c r="I41" s="8"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H42" s="10"/>
+      <c r="I42" s="8"/>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H43" s="10"/>
+      <c r="I43" s="8"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H44" s="10"/>
+      <c r="I44" s="8"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H45" s="10"/>
+      <c r="I45" s="8"/>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H46" s="10"/>
+      <c r="I46" s="8"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H47" s="10"/>
+      <c r="I47" s="8"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H48" s="10"/>
+      <c r="I48" s="8"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H49" s="10"/>
+      <c r="I49" s="8"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H50" s="10"/>
+      <c r="I50" s="8"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H51" s="10"/>
+      <c r="I51" s="8"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H52" s="10"/>
+      <c r="I52" s="8"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H53" s="10"/>
+      <c r="I53" s="8"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H54" s="10"/>
+      <c r="I54" s="8"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H55" s="10"/>
+      <c r="I55" s="8"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H56" s="10"/>
+      <c r="I56" s="8"/>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H57" s="10"/>
+      <c r="I57" s="8"/>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H58" s="10"/>
+      <c r="I58" s="8"/>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H59" s="10"/>
+      <c r="I59" s="8"/>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H60" s="10"/>
+      <c r="I60" s="8"/>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H61" s="10"/>
+      <c r="I61" s="8"/>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H62" s="10"/>
+      <c r="I62" s="8"/>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H63" s="10"/>
+      <c r="I63" s="8"/>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H64" s="10"/>
+      <c r="I64" s="8"/>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H65" s="10"/>
+      <c r="I65" s="8"/>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H66" s="10"/>
+      <c r="I66" s="8"/>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H67" s="10"/>
+      <c r="I67" s="8"/>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H68" s="10"/>
+      <c r="I68" s="8"/>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H69" s="10"/>
+      <c r="I69" s="8"/>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H70" s="10"/>
+      <c r="I70" s="8"/>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H71" s="10"/>
+      <c r="I71" s="8"/>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H72" s="10"/>
+      <c r="I72" s="8"/>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H73" s="10"/>
+      <c r="I73" s="8"/>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H74" s="10"/>
+      <c r="I74" s="8"/>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H75" s="10"/>
+      <c r="I75" s="8"/>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H76" s="10"/>
+      <c r="I76" s="8"/>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H77" s="10"/>
+      <c r="I77" s="8"/>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H78" s="10"/>
+      <c r="I78" s="8"/>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H79" s="10"/>
+      <c r="I79" s="8"/>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H80" s="10"/>
+      <c r="I80" s="8"/>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H81" s="10"/>
+      <c r="I81" s="8"/>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H82" s="10"/>
+      <c r="I82" s="8"/>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H83" s="10"/>
+      <c r="I83" s="8"/>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H84" s="10"/>
+      <c r="I84" s="8"/>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H85" s="10"/>
+      <c r="I85" s="8"/>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H86" s="10"/>
+      <c r="I86" s="8"/>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H87" s="10"/>
+      <c r="I87" s="8"/>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H88" s="10"/>
+      <c r="I88" s="8"/>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H89" s="10"/>
+      <c r="I89" s="8"/>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H90" s="10"/>
+      <c r="I90" s="8"/>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H91" s="10"/>
+      <c r="I91" s="8"/>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H92" s="10"/>
+      <c r="I92" s="8"/>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H93" s="10"/>
+      <c r="I93" s="8"/>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H94" s="10"/>
+      <c r="I94" s="8"/>
     </row>
     <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H95" s="10"/>
+      <c r="I95" s="8"/>
     </row>
     <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H96" s="10"/>
+      <c r="I96" s="8"/>
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H97" s="10"/>
+      <c r="I97" s="8"/>
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H98" s="10"/>
+      <c r="I98" s="8"/>
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H99" s="10"/>
+      <c r="I99" s="8"/>
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H100" s="10"/>
+      <c r="I100" s="8"/>
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H101" s="10"/>
+      <c r="I101" s="8"/>
     </row>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H102" s="10"/>
+      <c r="I102" s="8"/>
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H103" s="10"/>
+      <c r="I103" s="8"/>
     </row>
     <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H104" s="10"/>
+      <c r="I104" s="8"/>
     </row>
     <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H105" s="10"/>
+      <c r="I105" s="8"/>
     </row>
     <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H106" s="10"/>
+      <c r="I106" s="8"/>
     </row>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H107" s="10"/>
+      <c r="I107" s="8"/>
     </row>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H108" s="10"/>
+      <c r="I108" s="8"/>
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H109" s="10"/>
+      <c r="I109" s="8"/>
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H110" s="10"/>
+      <c r="I110" s="8"/>
     </row>
     <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H111" s="10"/>
+      <c r="I111" s="8"/>
     </row>
     <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H112" s="10"/>
+      <c r="I112" s="8"/>
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H113" s="10"/>
+      <c r="I113" s="8"/>
     </row>
     <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H114" s="10"/>
+      <c r="I114" s="8"/>
     </row>
     <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H115" s="10"/>
+      <c r="I115" s="8"/>
     </row>
     <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H116" s="10"/>
+      <c r="I116" s="8"/>
     </row>
     <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H117" s="10"/>
+      <c r="I117" s="8"/>
     </row>
     <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H118" s="10"/>
+      <c r="I118" s="8"/>
     </row>
     <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H119" s="10"/>
+      <c r="I119" s="8"/>
     </row>
     <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H120" s="10"/>
+      <c r="I120" s="8"/>
     </row>
     <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H121" s="10"/>
+      <c r="I121" s="8"/>
     </row>
     <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H122" s="10"/>
+      <c r="I122" s="8"/>
     </row>
     <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H123" s="10"/>
+      <c r="I123" s="8"/>
     </row>
     <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H124" s="10"/>
+      <c r="I124" s="8"/>
     </row>
     <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H125" s="10"/>
+      <c r="I125" s="8"/>
     </row>
     <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H126" s="10"/>
+      <c r="I126" s="8"/>
     </row>
     <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H127" s="10"/>
+      <c r="I127" s="8"/>
     </row>
     <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H128" s="10"/>
+      <c r="I128" s="8"/>
     </row>
     <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H129" s="10"/>
+      <c r="I129" s="8"/>
     </row>
     <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H130" s="10"/>
+      <c r="I130" s="8"/>
     </row>
     <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H131" s="10"/>
+      <c r="I131" s="8"/>
     </row>
     <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H132" s="10"/>
+      <c r="I132" s="8"/>
     </row>
     <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H133" s="10"/>
+      <c r="I133" s="8"/>
     </row>
     <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H134" s="10"/>
+      <c r="I134" s="8"/>
     </row>
     <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H135" s="10"/>
+      <c r="I135" s="8"/>
     </row>
     <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H136" s="10"/>
+      <c r="I136" s="8"/>
     </row>
     <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H137" s="10"/>
+      <c r="I137" s="8"/>
     </row>
     <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H138" s="10"/>
+      <c r="I138" s="8"/>
     </row>
     <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H139" s="10"/>
+      <c r="I139" s="8"/>
     </row>
     <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H140" s="10"/>
+      <c r="I140" s="8"/>
     </row>
     <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H141" s="10"/>
+      <c r="I141" s="8"/>
     </row>
     <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H142" s="10"/>
+      <c r="I142" s="8"/>
     </row>
     <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H143" s="10"/>
+      <c r="I143" s="8"/>
     </row>
     <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H144" s="10"/>
+      <c r="I144" s="8"/>
     </row>
     <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H145" s="10"/>
+      <c r="I145" s="8"/>
     </row>
     <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H146" s="10"/>
+      <c r="I146" s="8"/>
     </row>
     <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H147" s="10"/>
+      <c r="I147" s="8"/>
     </row>
     <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H148" s="10"/>
+      <c r="I148" s="8"/>
     </row>
     <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H149" s="10"/>
+      <c r="I149" s="8"/>
     </row>
     <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H150" s="10"/>
+      <c r="I150" s="8"/>
     </row>
     <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H151" s="10"/>
+      <c r="I151" s="8"/>
     </row>
     <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H152" s="10"/>
+      <c r="I152" s="8"/>
     </row>
     <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H153" s="10"/>
+      <c r="I153" s="8"/>
     </row>
     <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H154" s="10"/>
+      <c r="I154" s="8"/>
     </row>
     <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H155" s="10"/>
+      <c r="I155" s="8"/>
     </row>
     <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H156" s="10"/>
+      <c r="I156" s="8"/>
     </row>
     <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H157" s="10"/>
+      <c r="I157" s="8"/>
     </row>
     <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H158" s="10"/>
+      <c r="I158" s="8"/>
     </row>
     <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H159" s="10"/>
+      <c r="I159" s="8"/>
     </row>
     <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H160" s="10"/>
+      <c r="I160" s="8"/>
     </row>
     <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H161" s="10"/>
+      <c r="I161" s="8"/>
     </row>
     <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H162" s="10"/>
+      <c r="I162" s="8"/>
     </row>
     <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H163" s="10"/>
+      <c r="I163" s="8"/>
     </row>
     <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H164" s="10"/>
+      <c r="I164" s="8"/>
     </row>
     <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H165" s="10"/>
+      <c r="I165" s="8"/>
     </row>
     <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H166" s="10"/>
+      <c r="I166" s="8"/>
     </row>
     <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H167" s="10"/>
+      <c r="I167" s="8"/>
     </row>
     <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H168" s="10"/>
+      <c r="I168" s="8"/>
     </row>
     <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H169" s="10"/>
+      <c r="I169" s="8"/>
     </row>
     <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H170" s="10"/>
+      <c r="I170" s="8"/>
     </row>
     <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H171" s="10"/>
+      <c r="I171" s="8"/>
     </row>
     <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H172" s="10"/>
+      <c r="I172" s="8"/>
     </row>
     <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H173" s="10"/>
+      <c r="I173" s="8"/>
     </row>
     <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H174" s="10"/>
+      <c r="I174" s="8"/>
     </row>
     <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H175" s="10"/>
+      <c r="I175" s="8"/>
     </row>
     <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H176" s="10"/>
+      <c r="I176" s="8"/>
     </row>
     <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H177" s="10"/>
+      <c r="I177" s="8"/>
     </row>
     <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H178" s="10"/>
+      <c r="I178" s="8"/>
     </row>
     <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H179" s="10"/>
+      <c r="I179" s="8"/>
     </row>
     <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H180" s="10"/>
+      <c r="I180" s="8"/>
     </row>
     <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H181" s="10"/>
+      <c r="I181" s="8"/>
     </row>
     <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H182" s="10"/>
+      <c r="I182" s="8"/>
     </row>
     <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H183" s="10"/>
+      <c r="I183" s="8"/>
     </row>
     <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H184" s="10"/>
+      <c r="I184" s="8"/>
     </row>
     <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H185" s="10"/>
+      <c r="I185" s="8"/>
     </row>
     <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H186" s="10"/>
+      <c r="I186" s="8"/>
     </row>
     <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H187" s="10"/>
+      <c r="I187" s="8"/>
     </row>
     <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H188" s="10"/>
+      <c r="I188" s="8"/>
     </row>
     <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H189" s="10"/>
+      <c r="I189" s="8"/>
     </row>
     <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H190" s="10"/>
+      <c r="I190" s="8"/>
     </row>
     <row r="191" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H191" s="10"/>
+      <c r="I191" s="8"/>
     </row>
     <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H192" s="10"/>
+      <c r="I192" s="8"/>
     </row>
     <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H193" s="10"/>
+      <c r="I193" s="8"/>
     </row>
     <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H194" s="10"/>
+      <c r="I194" s="8"/>
     </row>
     <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H195" s="10"/>
+      <c r="I195" s="8"/>
     </row>
     <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H196" s="10"/>
+      <c r="I196" s="8"/>
     </row>
     <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H197" s="10"/>
+      <c r="I197" s="8"/>
     </row>
     <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H198" s="10"/>
+      <c r="I198" s="8"/>
     </row>
     <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H199" s="10"/>
+      <c r="I199" s="8"/>
     </row>
     <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H200" s="10"/>
+      <c r="I200" s="8"/>
     </row>
     <row r="201" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H201" s="10"/>
+      <c r="I201" s="8"/>
     </row>
     <row r="202" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H202" s="10"/>
+      <c r="I202" s="8"/>
     </row>
     <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H203" s="10"/>
+      <c r="I203" s="8"/>
     </row>
     <row r="204" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H204" s="10"/>
+      <c r="I204" s="8"/>
     </row>
     <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H205" s="10"/>
+      <c r="I205" s="8"/>
     </row>
     <row r="206" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H206" s="10"/>
+      <c r="I206" s="8"/>
     </row>
     <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H207" s="10"/>
+      <c r="I207" s="8"/>
     </row>
     <row r="208" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H208" s="10"/>
+      <c r="I208" s="8"/>
     </row>
     <row r="209" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H209" s="10"/>
+      <c r="I209" s="8"/>
     </row>
     <row r="210" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H210" s="10"/>
+      <c r="I210" s="8"/>
     </row>
     <row r="211" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H211" s="10"/>
+      <c r="I211" s="8"/>
     </row>
     <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H212" s="10"/>
+      <c r="I212" s="8"/>
     </row>
     <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H213" s="10"/>
+      <c r="I213" s="8"/>
     </row>
     <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H214" s="10"/>
+      <c r="I214" s="8"/>
     </row>
     <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H215" s="10"/>
+      <c r="I215" s="8"/>
     </row>
     <row r="216" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H216" s="10"/>
+      <c r="I216" s="8"/>
     </row>
     <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H217" s="10"/>
+      <c r="I217" s="8"/>
     </row>
     <row r="218" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H218" s="10"/>
+      <c r="I218" s="8"/>
     </row>
     <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H219" s="10"/>
+      <c r="I219" s="8"/>
     </row>
     <row r="220" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H220" s="10"/>
+      <c r="I220" s="8"/>
     </row>
     <row r="221" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H221" s="10"/>
+      <c r="I221" s="8"/>
     </row>
     <row r="222" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H222" s="10"/>
+      <c r="I222" s="8"/>
     </row>
     <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H223" s="10"/>
+      <c r="I223" s="8"/>
     </row>
     <row r="224" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H224" s="10"/>
+      <c r="I224" s="8"/>
     </row>
     <row r="225" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H225" s="10"/>
+      <c r="I225" s="8"/>
     </row>
     <row r="226" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H226" s="10"/>
+      <c r="I226" s="8"/>
     </row>
     <row r="227" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H227" s="10"/>
+      <c r="I227" s="8"/>
     </row>
     <row r="228" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H228" s="10"/>
+      <c r="I228" s="8"/>
     </row>
     <row r="229" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H229" s="10"/>
+      <c r="I229" s="8"/>
     </row>
     <row r="230" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H230" s="10"/>
+      <c r="I230" s="8"/>
     </row>
     <row r="231" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H231" s="10"/>
+      <c r="I231" s="8"/>
     </row>
     <row r="232" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H232" s="10"/>
+      <c r="I232" s="8"/>
     </row>
     <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H233" s="10"/>
+      <c r="I233" s="8"/>
     </row>
     <row r="234" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H234" s="10"/>
+      <c r="I234" s="8"/>
     </row>
     <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H235" s="10"/>
+      <c r="I235" s="8"/>
     </row>
     <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H236" s="10"/>
+      <c r="I236" s="8"/>
     </row>
     <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H237" s="10"/>
+      <c r="I237" s="8"/>
     </row>
     <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H238" s="10"/>
+      <c r="I238" s="8"/>
     </row>
     <row r="239" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H239" s="10"/>
+      <c r="I239" s="8"/>
     </row>
     <row r="240" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H240" s="10"/>
+      <c r="I240" s="8"/>
     </row>
     <row r="241" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H241" s="10"/>
+      <c r="I241" s="8"/>
     </row>
     <row r="242" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H242" s="10"/>
+      <c r="I242" s="8"/>
     </row>
     <row r="243" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H243" s="10"/>
+      <c r="I243" s="8"/>
     </row>
     <row r="244" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H244" s="10"/>
+      <c r="I244" s="8"/>
     </row>
     <row r="245" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H245" s="10"/>
+      <c r="I245" s="8"/>
     </row>
     <row r="246" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H246" s="10"/>
+      <c r="I246" s="8"/>
     </row>
     <row r="247" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H247" s="10"/>
+      <c r="I247" s="8"/>
     </row>
     <row r="248" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H248" s="10"/>
+      <c r="I248" s="8"/>
     </row>
     <row r="249" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H249" s="10"/>
+      <c r="I249" s="8"/>
     </row>
     <row r="250" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H250" s="10"/>
+      <c r="I250" s="8"/>
     </row>
     <row r="251" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H251" s="10"/>
+      <c r="I251" s="8"/>
     </row>
     <row r="252" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H252" s="10"/>
+      <c r="I252" s="8"/>
     </row>
     <row r="253" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H253" s="10"/>
+      <c r="I253" s="8"/>
     </row>
     <row r="254" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H254" s="10"/>
+      <c r="I254" s="8"/>
     </row>
     <row r="255" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H255" s="10"/>
+      <c r="I255" s="8"/>
     </row>
     <row r="256" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H256" s="10"/>
+      <c r="I256" s="8"/>
     </row>
     <row r="257" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H257" s="10"/>
+      <c r="I257" s="8"/>
     </row>
     <row r="258" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H258" s="10"/>
+      <c r="I258" s="8"/>
     </row>
     <row r="259" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H259" s="10"/>
+      <c r="I259" s="8"/>
     </row>
     <row r="260" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H260" s="10"/>
+      <c r="I260" s="8"/>
     </row>
     <row r="261" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H261" s="10"/>
+      <c r="I261" s="8"/>
     </row>
     <row r="262" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H262" s="10"/>
+      <c r="I262" s="8"/>
     </row>
     <row r="263" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H263" s="10"/>
+      <c r="I263" s="8"/>
     </row>
     <row r="264" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H264" s="10"/>
+      <c r="I264" s="8"/>
     </row>
     <row r="265" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H265" s="10"/>
+      <c r="I265" s="8"/>
     </row>
     <row r="266" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H266" s="10"/>
+      <c r="I266" s="8"/>
     </row>
     <row r="267" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H267" s="10"/>
+      <c r="I267" s="8"/>
     </row>
     <row r="268" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H268" s="10"/>
+      <c r="I268" s="8"/>
     </row>
     <row r="269" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H269" s="10"/>
+      <c r="I269" s="8"/>
     </row>
     <row r="270" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H270" s="10"/>
+      <c r="I270" s="8"/>
     </row>
     <row r="271" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H271" s="10"/>
+      <c r="I271" s="8"/>
     </row>
     <row r="272" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H272" s="10"/>
+      <c r="I272" s="8"/>
     </row>
     <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H273" s="10"/>
+      <c r="I273" s="8"/>
     </row>
     <row r="274" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H274" s="10"/>
+      <c r="I274" s="8"/>
     </row>
     <row r="275" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H275" s="10"/>
+      <c r="I275" s="8"/>
     </row>
     <row r="276" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H276" s="10"/>
+      <c r="I276" s="8"/>
     </row>
     <row r="277" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H277" s="10"/>
+      <c r="I277" s="8"/>
     </row>
     <row r="278" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H278" s="10"/>
+      <c r="I278" s="8"/>
     </row>
     <row r="279" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H279" s="10"/>
+      <c r="I279" s="8"/>
     </row>
     <row r="280" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H280" s="10"/>
+      <c r="I280" s="8"/>
     </row>
     <row r="281" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H281" s="10"/>
+      <c r="I281" s="8"/>
     </row>
     <row r="282" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H282" s="10"/>
+      <c r="I282" s="8"/>
     </row>
     <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H283" s="10"/>
+      <c r="I283" s="8"/>
     </row>
     <row r="284" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H284" s="10"/>
+      <c r="I284" s="8"/>
     </row>
     <row r="285" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H285" s="10"/>
+      <c r="I285" s="8"/>
     </row>
     <row r="286" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H286" s="10"/>
+      <c r="I286" s="8"/>
     </row>
     <row r="287" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H287" s="10"/>
+      <c r="I287" s="8"/>
     </row>
     <row r="288" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H288" s="10"/>
+      <c r="I288" s="8"/>
     </row>
     <row r="289" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H289" s="10"/>
+      <c r="I289" s="8"/>
     </row>
     <row r="290" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H290" s="10"/>
+      <c r="I290" s="8"/>
     </row>
     <row r="291" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H291" s="10"/>
+      <c r="I291" s="8"/>
     </row>
     <row r="292" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H292" s="10"/>
+      <c r="I292" s="8"/>
     </row>
     <row r="293" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H293" s="10"/>
+      <c r="I293" s="8"/>
     </row>
     <row r="294" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H294" s="10"/>
+      <c r="I294" s="8"/>
     </row>
     <row r="295" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H295" s="10"/>
+      <c r="I295" s="8"/>
     </row>
     <row r="296" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H296" s="10"/>
+      <c r="I296" s="8"/>
     </row>
     <row r="297" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H297" s="10"/>
+      <c r="I297" s="8"/>
     </row>
     <row r="298" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H298" s="10"/>
+      <c r="I298" s="8"/>
     </row>
     <row r="299" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H299" s="10"/>
+      <c r="I299" s="8"/>
     </row>
     <row r="300" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H300" s="10"/>
+      <c r="I300" s="8"/>
     </row>
     <row r="301" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H301" s="10"/>
+      <c r="I301" s="8"/>
     </row>
     <row r="302" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H302" s="10"/>
+      <c r="I302" s="8"/>
     </row>
     <row r="303" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H303" s="10"/>
+      <c r="I303" s="8"/>
     </row>
     <row r="304" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H304" s="10"/>
+      <c r="I304" s="8"/>
     </row>
     <row r="305" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H305" s="10"/>
+      <c r="I305" s="8"/>
     </row>
     <row r="306" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H306" s="10"/>
+      <c r="I306" s="8"/>
     </row>
     <row r="307" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H307" s="10"/>
+      <c r="I307" s="8"/>
     </row>
     <row r="308" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H308" s="10"/>
+      <c r="I308" s="8"/>
     </row>
     <row r="309" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H309" s="10"/>
+      <c r="I309" s="8"/>
     </row>
     <row r="310" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H310" s="10"/>
+      <c r="I310" s="8"/>
     </row>
     <row r="311" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H311" s="10"/>
+      <c r="I311" s="8"/>
     </row>
     <row r="312" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H312" s="10"/>
+      <c r="I312" s="8"/>
     </row>
     <row r="313" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H313" s="10"/>
+      <c r="I313" s="8"/>
     </row>
     <row r="314" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H314" s="10"/>
+      <c r="I314" s="8"/>
     </row>
     <row r="315" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H315" s="10"/>
+      <c r="I315" s="8"/>
     </row>
     <row r="316" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H316" s="10"/>
+      <c r="I316" s="8"/>
     </row>
     <row r="317" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H317" s="10"/>
+      <c r="I317" s="8"/>
     </row>
     <row r="318" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H318" s="10"/>
+      <c r="I318" s="8"/>
     </row>
     <row r="319" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H319" s="10"/>
+      <c r="I319" s="8"/>
     </row>
     <row r="320" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H320" s="10"/>
+      <c r="I320" s="8"/>
     </row>
     <row r="321" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H321" s="10"/>
+      <c r="I321" s="8"/>
     </row>
     <row r="322" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H322" s="10"/>
+      <c r="I322" s="8"/>
     </row>
     <row r="323" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H323" s="10"/>
+      <c r="I323" s="8"/>
     </row>
     <row r="324" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H324" s="10"/>
+      <c r="I324" s="8"/>
     </row>
     <row r="325" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H325" s="10"/>
+      <c r="I325" s="8"/>
     </row>
     <row r="326" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H326" s="10"/>
+      <c r="I326" s="8"/>
     </row>
     <row r="327" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H327" s="10"/>
+      <c r="I327" s="8"/>
     </row>
     <row r="328" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H328" s="10"/>
+      <c r="I328" s="8"/>
     </row>
     <row r="329" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H329" s="10"/>
+      <c r="I329" s="8"/>
     </row>
     <row r="330" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H330" s="10"/>
+      <c r="I330" s="8"/>
     </row>
     <row r="331" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H331" s="10"/>
+      <c r="I331" s="8"/>
     </row>
     <row r="332" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H332" s="10"/>
+      <c r="I332" s="8"/>
     </row>
     <row r="333" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H333" s="10"/>
+      <c r="I333" s="8"/>
     </row>
     <row r="334" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H334" s="10"/>
+      <c r="I334" s="8"/>
     </row>
     <row r="335" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H335" s="10"/>
+      <c r="I335" s="8"/>
     </row>
     <row r="336" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H336" s="10"/>
+      <c r="I336" s="8"/>
     </row>
     <row r="337" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H337" s="10"/>
+      <c r="I337" s="8"/>
     </row>
     <row r="338" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H338" s="10"/>
+      <c r="I338" s="8"/>
     </row>
     <row r="339" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H339" s="10"/>
+      <c r="I339" s="8"/>
     </row>
     <row r="340" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H340" s="10"/>
+      <c r="I340" s="8"/>
     </row>
     <row r="341" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H341" s="10"/>
+      <c r="I341" s="8"/>
     </row>
     <row r="342" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H342" s="10"/>
+      <c r="I342" s="8"/>
     </row>
     <row r="343" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H343" s="10"/>
+      <c r="I343" s="8"/>
     </row>
     <row r="344" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H344" s="10"/>
+      <c r="I344" s="8"/>
     </row>
     <row r="345" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H345" s="10"/>
+      <c r="I345" s="8"/>
     </row>
     <row r="346" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H346" s="10"/>
+      <c r="I346" s="8"/>
     </row>
     <row r="347" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H347" s="10"/>
+      <c r="I347" s="8"/>
     </row>
     <row r="348" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H348" s="10"/>
+      <c r="I348" s="8"/>
     </row>
     <row r="349" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H349" s="10"/>
+      <c r="I349" s="8"/>
     </row>
     <row r="350" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H350" s="10"/>
+      <c r="I350" s="8"/>
     </row>
     <row r="351" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H351" s="10"/>
+      <c r="I351" s="8"/>
     </row>
     <row r="352" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H352" s="10"/>
+      <c r="I352" s="8"/>
     </row>
     <row r="353" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H353" s="10"/>
+      <c r="I353" s="8"/>
     </row>
     <row r="354" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H354" s="10"/>
+      <c r="I354" s="8"/>
     </row>
     <row r="355" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H355" s="10"/>
+      <c r="I355" s="8"/>
     </row>
     <row r="356" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H356" s="10"/>
+      <c r="I356" s="8"/>
     </row>
     <row r="357" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H357" s="10"/>
+      <c r="I357" s="8"/>
     </row>
     <row r="358" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H358" s="10"/>
+      <c r="I358" s="8"/>
     </row>
     <row r="359" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H359" s="10"/>
+      <c r="I359" s="8"/>
     </row>
     <row r="360" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H360" s="10"/>
+      <c r="I360" s="8"/>
     </row>
     <row r="361" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H361" s="10"/>
+      <c r="I361" s="8"/>
     </row>
     <row r="362" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H362" s="10"/>
+      <c r="I362" s="8"/>
     </row>
     <row r="363" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H363" s="10"/>
+      <c r="I363" s="8"/>
     </row>
     <row r="364" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H364" s="10"/>
+      <c r="I364" s="8"/>
     </row>
     <row r="365" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H365" s="10"/>
+      <c r="I365" s="8"/>
     </row>
     <row r="366" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H366" s="10"/>
+      <c r="I366" s="8"/>
     </row>
     <row r="367" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H367" s="10"/>
+      <c r="I367" s="8"/>
     </row>
     <row r="368" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H368" s="10"/>
+      <c r="I368" s="8"/>
     </row>
     <row r="369" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H369" s="10"/>
+      <c r="I369" s="8"/>
     </row>
     <row r="370" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H370" s="10"/>
+      <c r="I370" s="8"/>
     </row>
     <row r="371" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H371" s="10"/>
+      <c r="I371" s="8"/>
     </row>
     <row r="372" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H372" s="10"/>
+      <c r="I372" s="8"/>
     </row>
     <row r="373" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H373" s="10"/>
+      <c r="I373" s="8"/>
     </row>
     <row r="374" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H374" s="10"/>
+      <c r="I374" s="8"/>
     </row>
     <row r="375" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H375" s="10"/>
+      <c r="I375" s="8"/>
     </row>
     <row r="376" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H376" s="10"/>
+      <c r="I376" s="8"/>
     </row>
     <row r="377" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H377" s="10"/>
+      <c r="I377" s="8"/>
     </row>
     <row r="378" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H378" s="10"/>
+      <c r="I378" s="8"/>
     </row>
     <row r="379" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H379" s="10"/>
+      <c r="I379" s="8"/>
     </row>
     <row r="380" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H380" s="10"/>
+      <c r="I380" s="8"/>
     </row>
     <row r="381" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H381" s="10"/>
+      <c r="I381" s="8"/>
     </row>
     <row r="382" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H382" s="10"/>
+      <c r="I382" s="8"/>
     </row>
     <row r="383" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H383" s="10"/>
+      <c r="I383" s="8"/>
     </row>
     <row r="384" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H384" s="10"/>
+      <c r="I384" s="8"/>
     </row>
     <row r="385" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H385" s="10"/>
+      <c r="I385" s="8"/>
     </row>
     <row r="386" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H386" s="10"/>
+      <c r="I386" s="8"/>
     </row>
     <row r="387" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H387" s="10"/>
+      <c r="I387" s="8"/>
     </row>
     <row r="388" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H388" s="10"/>
+      <c r="I388" s="8"/>
     </row>
     <row r="389" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H389" s="10"/>
+      <c r="I389" s="8"/>
     </row>
     <row r="390" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H390" s="10"/>
+      <c r="I390" s="8"/>
     </row>
     <row r="391" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H391" s="10"/>
+      <c r="I391" s="8"/>
     </row>
     <row r="392" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H392" s="10"/>
+      <c r="I392" s="8"/>
     </row>
     <row r="393" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H393" s="10"/>
+      <c r="I393" s="8"/>
     </row>
     <row r="394" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H394" s="10"/>
+      <c r="I394" s="8"/>
     </row>
     <row r="395" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H395" s="10"/>
+      <c r="I395" s="8"/>
     </row>
     <row r="396" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H396" s="10"/>
+      <c r="I396" s="8"/>
     </row>
     <row r="397" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H397" s="10"/>
+      <c r="I397" s="8"/>
     </row>
     <row r="398" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H398" s="10"/>
+      <c r="I398" s="8"/>
     </row>
     <row r="399" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H399" s="10"/>
+      <c r="I399" s="8"/>
     </row>
     <row r="400" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H400" s="10"/>
+      <c r="I400" s="8"/>
     </row>
     <row r="401" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H401" s="10"/>
+      <c r="I401" s="8"/>
     </row>
     <row r="402" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H402" s="10"/>
+      <c r="I402" s="8"/>
     </row>
     <row r="403" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H403" s="10"/>
+      <c r="I403" s="8"/>
     </row>
     <row r="404" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H404" s="10"/>
+      <c r="I404" s="8"/>
     </row>
     <row r="405" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H405" s="10"/>
+      <c r="I405" s="8"/>
     </row>
     <row r="406" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H406" s="10"/>
+      <c r="I406" s="8"/>
     </row>
     <row r="407" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H407" s="10"/>
+      <c r="I407" s="8"/>
     </row>
     <row r="408" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H408" s="10"/>
+      <c r="I408" s="8"/>
     </row>
     <row r="409" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H409" s="10"/>
+      <c r="I409" s="8"/>
     </row>
     <row r="410" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H410" s="10"/>
+      <c r="I410" s="8"/>
     </row>
     <row r="411" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H411" s="10"/>
+      <c r="I411" s="8"/>
     </row>
     <row r="412" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H412" s="10"/>
+      <c r="I412" s="8"/>
     </row>
     <row r="413" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H413" s="10"/>
+      <c r="I413" s="8"/>
     </row>
     <row r="414" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H414" s="10"/>
+      <c r="I414" s="8"/>
     </row>
     <row r="415" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H415" s="10"/>
+      <c r="I415" s="8"/>
     </row>
     <row r="416" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H416" s="10"/>
+      <c r="I416" s="8"/>
     </row>
     <row r="417" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H417" s="10"/>
+      <c r="I417" s="8"/>
     </row>
     <row r="418" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H418" s="10"/>
+      <c r="I418" s="8"/>
     </row>
     <row r="419" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H419" s="10"/>
+      <c r="I419" s="8"/>
     </row>
     <row r="420" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H420" s="10"/>
+      <c r="I420" s="8"/>
     </row>
     <row r="421" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H421" s="10"/>
+      <c r="I421" s="8"/>
     </row>
     <row r="422" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H422" s="10"/>
+      <c r="I422" s="8"/>
     </row>
     <row r="423" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H423" s="10"/>
+      <c r="I423" s="8"/>
     </row>
     <row r="424" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H424" s="10"/>
+      <c r="I424" s="8"/>
     </row>
     <row r="425" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H425" s="10"/>
+      <c r="I425" s="8"/>
     </row>
     <row r="426" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H426" s="10"/>
+      <c r="I426" s="8"/>
     </row>
     <row r="427" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H427" s="10"/>
+      <c r="I427" s="8"/>
     </row>
     <row r="428" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H428" s="10"/>
+      <c r="I428" s="8"/>
     </row>
     <row r="429" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H429" s="10"/>
+      <c r="I429" s="8"/>
     </row>
     <row r="430" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H430" s="10"/>
+      <c r="I430" s="8"/>
     </row>
     <row r="431" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H431" s="10"/>
+      <c r="I431" s="8"/>
     </row>
     <row r="432" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H432" s="10"/>
+      <c r="I432" s="8"/>
     </row>
     <row r="433" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H433" s="10"/>
+      <c r="I433" s="8"/>
     </row>
     <row r="434" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H434" s="10"/>
+      <c r="I434" s="8"/>
     </row>
     <row r="435" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H435" s="10"/>
+      <c r="I435" s="8"/>
     </row>
     <row r="436" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H436" s="10"/>
+      <c r="I436" s="8"/>
     </row>
     <row r="437" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H437" s="10"/>
+      <c r="I437" s="8"/>
     </row>
     <row r="438" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H438" s="10"/>
+      <c r="I438" s="8"/>
     </row>
     <row r="439" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H439" s="10"/>
+      <c r="I439" s="8"/>
     </row>
     <row r="440" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H440" s="10"/>
+      <c r="I440" s="8"/>
     </row>
     <row r="441" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H441" s="10"/>
+      <c r="I441" s="8"/>
     </row>
     <row r="442" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H442" s="10"/>
+      <c r="I442" s="8"/>
     </row>
     <row r="443" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H443" s="10"/>
+      <c r="I443" s="8"/>
     </row>
     <row r="444" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H444" s="10"/>
+      <c r="I444" s="8"/>
     </row>
     <row r="445" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H445" s="10"/>
+      <c r="I445" s="8"/>
     </row>
     <row r="446" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H446" s="10"/>
+      <c r="I446" s="8"/>
     </row>
     <row r="447" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H447" s="10"/>
+      <c r="I447" s="8"/>
     </row>
     <row r="448" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H448" s="10"/>
+      <c r="I448" s="8"/>
     </row>
     <row r="449" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H449" s="10"/>
+      <c r="I449" s="8"/>
     </row>
     <row r="450" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H450" s="10"/>
+      <c r="I450" s="8"/>
     </row>
     <row r="451" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H451" s="10"/>
+      <c r="I451" s="8"/>
     </row>
     <row r="452" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H452" s="10"/>
+      <c r="I452" s="8"/>
     </row>
     <row r="453" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H453" s="10"/>
+      <c r="I453" s="8"/>
     </row>
     <row r="454" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H454" s="10"/>
+      <c r="I454" s="8"/>
     </row>
     <row r="455" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H455" s="10"/>
+      <c r="I455" s="8"/>
     </row>
     <row r="456" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H456" s="10"/>
+      <c r="I456" s="8"/>
     </row>
     <row r="457" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H457" s="10"/>
+      <c r="I457" s="8"/>
     </row>
     <row r="458" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H458" s="10"/>
+      <c r="I458" s="8"/>
     </row>
     <row r="459" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H459" s="10"/>
+      <c r="I459" s="8"/>
     </row>
     <row r="460" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H460" s="10"/>
+      <c r="I460" s="8"/>
     </row>
     <row r="461" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H461" s="10"/>
+      <c r="I461" s="8"/>
     </row>
     <row r="462" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H462" s="10"/>
+      <c r="I462" s="8"/>
     </row>
     <row r="463" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H463" s="10"/>
+      <c r="I463" s="8"/>
     </row>
     <row r="464" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H464" s="10"/>
+      <c r="I464" s="8"/>
     </row>
     <row r="465" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H465" s="10"/>
+      <c r="I465" s="8"/>
     </row>
     <row r="466" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H466" s="10"/>
+      <c r="I466" s="8"/>
     </row>
     <row r="467" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H467" s="10"/>
+      <c r="I467" s="8"/>
     </row>
     <row r="468" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H468" s="10"/>
+      <c r="I468" s="8"/>
     </row>
     <row r="469" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H469" s="10"/>
+      <c r="I469" s="8"/>
     </row>
     <row r="470" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H470" s="10"/>
+      <c r="I470" s="8"/>
     </row>
     <row r="471" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H471" s="10"/>
+      <c r="I471" s="8"/>
     </row>
     <row r="472" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H472" s="10"/>
+      <c r="I472" s="8"/>
     </row>
     <row r="473" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H473" s="10"/>
+      <c r="I473" s="8"/>
     </row>
     <row r="474" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H474" s="10"/>
+      <c r="I474" s="8"/>
     </row>
     <row r="475" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H475" s="10"/>
+      <c r="I475" s="8"/>
     </row>
     <row r="476" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H476" s="10"/>
+      <c r="I476" s="8"/>
     </row>
     <row r="477" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H477" s="10"/>
+      <c r="I477" s="8"/>
     </row>
     <row r="478" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H478" s="10"/>
+      <c r="I478" s="8"/>
     </row>
     <row r="479" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H479" s="10"/>
+      <c r="I479" s="8"/>
     </row>
     <row r="480" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H480" s="10"/>
+      <c r="I480" s="8"/>
     </row>
     <row r="481" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H481" s="10"/>
+      <c r="I481" s="8"/>
     </row>
     <row r="482" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H482" s="10"/>
+      <c r="I482" s="8"/>
     </row>
     <row r="483" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H483" s="10"/>
+      <c r="I483" s="8"/>
     </row>
     <row r="484" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H484" s="10"/>
+      <c r="I484" s="8"/>
     </row>
     <row r="485" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H485" s="10"/>
+      <c r="I485" s="8"/>
     </row>
     <row r="486" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H486" s="10"/>
+      <c r="I486" s="8"/>
     </row>
     <row r="487" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H487" s="10"/>
+      <c r="I487" s="8"/>
     </row>
     <row r="488" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H488" s="10"/>
+      <c r="I488" s="8"/>
     </row>
     <row r="489" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H489" s="10"/>
+      <c r="I489" s="8"/>
     </row>
     <row r="490" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H490" s="10"/>
+      <c r="I490" s="8"/>
     </row>
     <row r="491" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H491" s="10"/>
+      <c r="I491" s="8"/>
     </row>
     <row r="492" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H492" s="10"/>
+      <c r="I492" s="8"/>
     </row>
     <row r="493" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H493" s="10"/>
+      <c r="I493" s="8"/>
     </row>
     <row r="494" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H494" s="10"/>
+      <c r="I494" s="8"/>
     </row>
     <row r="495" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H495" s="10"/>
+      <c r="I495" s="8"/>
     </row>
     <row r="496" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H496" s="10"/>
+      <c r="I496" s="8"/>
     </row>
     <row r="497" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H497" s="10"/>
+      <c r="I497" s="8"/>
     </row>
     <row r="498" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H498" s="10"/>
+      <c r="I498" s="8"/>
     </row>
     <row r="499" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H499" s="10"/>
+      <c r="I499" s="8"/>
     </row>
     <row r="500" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H500" s="10"/>
+      <c r="I500" s="8"/>
     </row>
     <row r="501" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H501" s="10"/>
+      <c r="I501" s="8"/>
     </row>
     <row r="502" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H502" s="10"/>
+      <c r="I502" s="8"/>
     </row>
     <row r="503" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H503" s="10"/>
+      <c r="I503" s="8"/>
     </row>
     <row r="504" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H504" s="10"/>
+      <c r="I504" s="8"/>
     </row>
     <row r="505" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H505" s="10"/>
+      <c r="I505" s="8"/>
     </row>
     <row r="506" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H506" s="10"/>
+      <c r="I506" s="8"/>
     </row>
     <row r="507" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H507" s="10"/>
+      <c r="I507" s="8"/>
     </row>
     <row r="508" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H508" s="10"/>
+      <c r="I508" s="8"/>
     </row>
     <row r="509" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H509" s="10"/>
+      <c r="I509" s="8"/>
     </row>
     <row r="510" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H510" s="10"/>
+      <c r="I510" s="8"/>
     </row>
     <row r="511" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H511" s="10"/>
+      <c r="I511" s="8"/>
     </row>
     <row r="512" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H512" s="10"/>
+      <c r="I512" s="8"/>
     </row>
     <row r="513" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H513" s="10"/>
+      <c r="I513" s="8"/>
     </row>
     <row r="514" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H514" s="10"/>
+      <c r="I514" s="8"/>
     </row>
     <row r="515" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H515" s="10"/>
+      <c r="I515" s="8"/>
     </row>
     <row r="516" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H516" s="10"/>
+      <c r="I516" s="8"/>
     </row>
     <row r="517" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H517" s="10"/>
+      <c r="I517" s="8"/>
     </row>
     <row r="518" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H518" s="10"/>
+      <c r="I518" s="8"/>
     </row>
     <row r="519" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H519" s="10"/>
+      <c r="I519" s="8"/>
     </row>
     <row r="520" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H520" s="10"/>
+      <c r="I520" s="8"/>
     </row>
     <row r="521" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H521" s="10"/>
+      <c r="I521" s="8"/>
     </row>
     <row r="522" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H522" s="10"/>
+      <c r="I522" s="8"/>
     </row>
     <row r="523" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H523" s="10"/>
+      <c r="I523" s="8"/>
     </row>
     <row r="524" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H524" s="10"/>
+      <c r="I524" s="8"/>
     </row>
     <row r="525" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H525" s="10"/>
+      <c r="I525" s="8"/>
     </row>
     <row r="526" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H526" s="10"/>
+      <c r="I526" s="8"/>
     </row>
     <row r="527" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H527" s="10"/>
+      <c r="I527" s="8"/>
     </row>
     <row r="528" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H528" s="10"/>
+      <c r="I528" s="8"/>
     </row>
     <row r="529" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H529" s="10"/>
+      <c r="I529" s="8"/>
     </row>
     <row r="530" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H530" s="10"/>
+      <c r="I530" s="8"/>
     </row>
     <row r="531" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H531" s="10"/>
+      <c r="I531" s="8"/>
     </row>
     <row r="532" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H532" s="10"/>
+      <c r="I532" s="8"/>
     </row>
     <row r="533" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H533" s="10"/>
+      <c r="I533" s="8"/>
     </row>
     <row r="534" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H534" s="10"/>
+      <c r="I534" s="8"/>
     </row>
     <row r="535" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H535" s="10"/>
+      <c r="I535" s="8"/>
     </row>
     <row r="536" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H536" s="10"/>
+      <c r="I536" s="8"/>
     </row>
     <row r="537" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H537" s="10"/>
+      <c r="I537" s="8"/>
     </row>
     <row r="538" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H538" s="10"/>
+      <c r="I538" s="8"/>
     </row>
     <row r="539" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H539" s="10"/>
+      <c r="I539" s="8"/>
     </row>
     <row r="540" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H540" s="10"/>
+      <c r="I540" s="8"/>
     </row>
     <row r="541" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H541" s="10"/>
+      <c r="I541" s="8"/>
     </row>
     <row r="542" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H542" s="10"/>
+      <c r="I542" s="8"/>
     </row>
     <row r="543" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H543" s="10"/>
+      <c r="I543" s="8"/>
     </row>
     <row r="544" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H544" s="10"/>
+      <c r="I544" s="8"/>
     </row>
     <row r="545" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H545" s="10"/>
+      <c r="I545" s="8"/>
     </row>
     <row r="546" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H546" s="10"/>
+      <c r="I546" s="8"/>
     </row>
     <row r="547" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H547" s="10"/>
+      <c r="I547" s="8"/>
     </row>
     <row r="548" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H548" s="10"/>
+      <c r="I548" s="8"/>
     </row>
     <row r="549" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H549" s="10"/>
+      <c r="I549" s="8"/>
     </row>
     <row r="550" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H550" s="10"/>
+      <c r="I550" s="8"/>
     </row>
     <row r="551" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H551" s="10"/>
+      <c r="I551" s="8"/>
     </row>
     <row r="552" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H552" s="10"/>
+      <c r="I552" s="8"/>
     </row>
     <row r="553" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H553" s="10"/>
+      <c r="I553" s="8"/>
     </row>
     <row r="554" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H554" s="10"/>
+      <c r="I554" s="8"/>
     </row>
     <row r="555" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H555" s="10"/>
+      <c r="I555" s="8"/>
     </row>
     <row r="556" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H556" s="10"/>
+      <c r="I556" s="8"/>
     </row>
     <row r="557" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H557" s="10"/>
+      <c r="I557" s="8"/>
     </row>
     <row r="558" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H558" s="10"/>
+      <c r="I558" s="8"/>
     </row>
     <row r="559" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H559" s="10"/>
+      <c r="I559" s="8"/>
     </row>
     <row r="560" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H560" s="10"/>
+      <c r="I560" s="8"/>
     </row>
     <row r="561" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H561" s="10"/>
+      <c r="I561" s="8"/>
     </row>
     <row r="562" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H562" s="10"/>
+      <c r="I562" s="8"/>
     </row>
     <row r="563" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H563" s="10"/>
+      <c r="I563" s="8"/>
     </row>
     <row r="564" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H564" s="10"/>
+      <c r="I564" s="8"/>
     </row>
     <row r="565" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H565" s="10"/>
+      <c r="I565" s="8"/>
     </row>
     <row r="566" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H566" s="10"/>
+      <c r="I566" s="8"/>
     </row>
     <row r="567" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H567" s="10"/>
+      <c r="I567" s="8"/>
     </row>
     <row r="568" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H568" s="10"/>
+      <c r="I568" s="8"/>
     </row>
     <row r="569" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H569" s="10"/>
+      <c r="I569" s="8"/>
     </row>
     <row r="570" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H570" s="10"/>
+      <c r="I570" s="8"/>
     </row>
     <row r="571" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H571" s="10"/>
+      <c r="I571" s="8"/>
     </row>
     <row r="572" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H572" s="10"/>
+      <c r="I572" s="8"/>
     </row>
     <row r="573" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H573" s="10"/>
+      <c r="I573" s="8"/>
     </row>
     <row r="574" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H574" s="10"/>
+      <c r="I574" s="8"/>
     </row>
     <row r="575" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H575" s="10"/>
+      <c r="I575" s="8"/>
     </row>
     <row r="576" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H576" s="10"/>
+      <c r="I576" s="8"/>
     </row>
     <row r="577" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H577" s="10"/>
+      <c r="I577" s="8"/>
     </row>
     <row r="578" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H578" s="10"/>
+      <c r="I578" s="8"/>
     </row>
     <row r="579" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H579" s="10"/>
+      <c r="I579" s="8"/>
     </row>
     <row r="580" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H580" s="10"/>
+      <c r="I580" s="8"/>
     </row>
     <row r="581" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H581" s="10"/>
+      <c r="I581" s="8"/>
     </row>
     <row r="582" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H582" s="10"/>
+      <c r="I582" s="8"/>
     </row>
     <row r="583" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H583" s="10"/>
+      <c r="I583" s="8"/>
     </row>
     <row r="584" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H584" s="10"/>
+      <c r="I584" s="8"/>
     </row>
     <row r="585" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H585" s="10"/>
+      <c r="I585" s="8"/>
     </row>
     <row r="586" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H586" s="10"/>
+      <c r="I586" s="8"/>
     </row>
     <row r="587" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H587" s="10"/>
+      <c r="I587" s="8"/>
     </row>
     <row r="588" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H588" s="10"/>
+      <c r="I588" s="8"/>
     </row>
     <row r="589" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H589" s="10"/>
+      <c r="I589" s="8"/>
     </row>
     <row r="590" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H590" s="10"/>
+      <c r="I590" s="8"/>
     </row>
     <row r="591" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H591" s="10"/>
+      <c r="I591" s="8"/>
     </row>
     <row r="592" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H592" s="10"/>
+      <c r="I592" s="8"/>
     </row>
     <row r="593" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H593" s="10"/>
+      <c r="I593" s="8"/>
     </row>
     <row r="594" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H594" s="10"/>
+      <c r="I594" s="8"/>
     </row>
     <row r="595" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H595" s="10"/>
+      <c r="I595" s="8"/>
     </row>
     <row r="596" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H596" s="10"/>
+      <c r="I596" s="8"/>
     </row>
     <row r="597" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H597" s="10"/>
+      <c r="I597" s="8"/>
     </row>
     <row r="598" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H598" s="10"/>
+      <c r="I598" s="8"/>
     </row>
     <row r="599" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H599" s="10"/>
+      <c r="I599" s="8"/>
     </row>
     <row r="600" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H600" s="10"/>
+      <c r="I600" s="8"/>
     </row>
     <row r="601" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H601" s="10"/>
+      <c r="I601" s="8"/>
     </row>
     <row r="602" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H602" s="10"/>
+      <c r="I602" s="8"/>
     </row>
     <row r="603" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H603" s="10"/>
+      <c r="I603" s="8"/>
     </row>
     <row r="604" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H604" s="10"/>
+      <c r="I604" s="8"/>
     </row>
     <row r="605" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H605" s="10"/>
+      <c r="I605" s="8"/>
     </row>
     <row r="606" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H606" s="10"/>
+      <c r="I606" s="8"/>
     </row>
     <row r="607" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H607" s="10"/>
+      <c r="I607" s="8"/>
     </row>
     <row r="608" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H608" s="10"/>
+      <c r="I608" s="8"/>
     </row>
     <row r="609" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H609" s="10"/>
+      <c r="I609" s="8"/>
     </row>
     <row r="610" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H610" s="10"/>
+      <c r="I610" s="8"/>
     </row>
     <row r="611" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H611" s="10"/>
+      <c r="I611" s="8"/>
     </row>
     <row r="612" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H612" s="10"/>
+      <c r="I612" s="8"/>
     </row>
     <row r="613" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H613" s="10"/>
+      <c r="I613" s="8"/>
     </row>
     <row r="614" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H614" s="10"/>
+      <c r="I614" s="8"/>
     </row>
     <row r="615" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H615" s="10"/>
+      <c r="I615" s="8"/>
     </row>
     <row r="616" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H616" s="10"/>
+      <c r="I616" s="8"/>
     </row>
     <row r="617" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H617" s="10"/>
+      <c r="I617" s="8"/>
     </row>
     <row r="618" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H618" s="10"/>
+      <c r="I618" s="8"/>
     </row>
     <row r="619" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H619" s="10"/>
+      <c r="I619" s="8"/>
     </row>
     <row r="620" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H620" s="10"/>
+      <c r="I620" s="8"/>
     </row>
     <row r="621" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H621" s="10"/>
+      <c r="I621" s="8"/>
     </row>
     <row r="622" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H622" s="10"/>
+      <c r="I622" s="8"/>
     </row>
     <row r="623" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H623" s="10"/>
+      <c r="I623" s="8"/>
     </row>
     <row r="624" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H624" s="10"/>
+      <c r="I624" s="8"/>
     </row>
     <row r="625" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H625" s="10"/>
+      <c r="I625" s="8"/>
     </row>
     <row r="626" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H626" s="10"/>
+      <c r="I626" s="8"/>
     </row>
     <row r="627" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H627" s="10"/>
+      <c r="I627" s="8"/>
     </row>
     <row r="628" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H628" s="10"/>
+      <c r="I628" s="8"/>
     </row>
     <row r="629" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H629" s="10"/>
+      <c r="I629" s="8"/>
     </row>
     <row r="630" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H630" s="10"/>
+      <c r="I630" s="8"/>
     </row>
     <row r="631" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H631" s="10"/>
+      <c r="I631" s="8"/>
     </row>
     <row r="632" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H632" s="10"/>
+      <c r="I632" s="8"/>
     </row>
     <row r="633" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H633" s="10"/>
+      <c r="I633" s="8"/>
     </row>
     <row r="634" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H634" s="10"/>
+      <c r="I634" s="8"/>
     </row>
     <row r="635" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H635" s="10"/>
+      <c r="I635" s="8"/>
     </row>
     <row r="636" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H636" s="10"/>
+      <c r="I636" s="8"/>
     </row>
     <row r="637" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H637" s="10"/>
+      <c r="I637" s="8"/>
     </row>
     <row r="638" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H638" s="10"/>
+      <c r="I638" s="8"/>
     </row>
     <row r="639" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H639" s="10"/>
+      <c r="I639" s="8"/>
     </row>
     <row r="640" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H640" s="10"/>
+      <c r="I640" s="8"/>
     </row>
     <row r="641" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H641" s="10"/>
+      <c r="I641" s="8"/>
     </row>
     <row r="642" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H642" s="10"/>
+      <c r="I642" s="8"/>
     </row>
     <row r="643" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H643" s="10"/>
+      <c r="I643" s="8"/>
     </row>
     <row r="644" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H644" s="10"/>
+      <c r="I644" s="8"/>
     </row>
     <row r="645" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H645" s="10"/>
+      <c r="I645" s="8"/>
     </row>
     <row r="646" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H646" s="10"/>
+      <c r="I646" s="8"/>
     </row>
     <row r="647" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H647" s="10"/>
+      <c r="I647" s="8"/>
     </row>
     <row r="648" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H648" s="10"/>
+      <c r="I648" s="8"/>
     </row>
     <row r="649" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H649" s="10"/>
+      <c r="I649" s="8"/>
     </row>
     <row r="650" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H650" s="10"/>
+      <c r="I650" s="8"/>
     </row>
     <row r="651" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H651" s="10"/>
+      <c r="I651" s="8"/>
     </row>
     <row r="652" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H652" s="10"/>
+      <c r="I652" s="8"/>
     </row>
     <row r="653" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H653" s="10"/>
+      <c r="I653" s="8"/>
     </row>
     <row r="654" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H654" s="10"/>
+      <c r="I654" s="8"/>
     </row>
     <row r="655" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H655" s="10"/>
+      <c r="I655" s="8"/>
     </row>
     <row r="656" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H656" s="10"/>
+      <c r="I656" s="8"/>
     </row>
     <row r="657" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H657" s="10"/>
+      <c r="I657" s="8"/>
     </row>
     <row r="658" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H658" s="10"/>
+      <c r="I658" s="8"/>
     </row>
     <row r="659" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H659" s="10"/>
+      <c r="I659" s="8"/>
     </row>
     <row r="660" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H660" s="10"/>
+      <c r="I660" s="8"/>
     </row>
     <row r="661" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H661" s="10"/>
+      <c r="I661" s="8"/>
     </row>
     <row r="662" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H662" s="10"/>
+      <c r="I662" s="8"/>
     </row>
     <row r="663" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H663" s="10"/>
+      <c r="I663" s="8"/>
     </row>
     <row r="664" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H664" s="10"/>
+      <c r="I664" s="8"/>
     </row>
     <row r="665" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H665" s="10"/>
+      <c r="I665" s="8"/>
     </row>
     <row r="666" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H666" s="10"/>
+      <c r="I666" s="8"/>
     </row>
     <row r="667" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H667" s="10"/>
+      <c r="I667" s="8"/>
     </row>
     <row r="668" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H668" s="10"/>
+      <c r="I668" s="8"/>
     </row>
     <row r="669" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H669" s="10"/>
+      <c r="I669" s="8"/>
     </row>
     <row r="670" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H670" s="10"/>
+      <c r="I670" s="8"/>
     </row>
     <row r="671" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H671" s="10"/>
+      <c r="I671" s="8"/>
     </row>
     <row r="672" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H672" s="10"/>
+      <c r="I672" s="8"/>
     </row>
     <row r="673" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H673" s="10"/>
+      <c r="I673" s="8"/>
     </row>
     <row r="674" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H674" s="10"/>
+      <c r="I674" s="8"/>
     </row>
     <row r="675" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H675" s="10"/>
+      <c r="I675" s="8"/>
     </row>
     <row r="676" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H676" s="10"/>
+      <c r="I676" s="8"/>
     </row>
     <row r="677" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H677" s="10"/>
+      <c r="I677" s="8"/>
     </row>
     <row r="678" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H678" s="10"/>
+      <c r="I678" s="8"/>
     </row>
     <row r="679" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H679" s="10"/>
+      <c r="I679" s="8"/>
     </row>
     <row r="680" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H680" s="10"/>
+      <c r="I680" s="8"/>
     </row>
     <row r="681" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H681" s="10"/>
+      <c r="I681" s="8"/>
     </row>
     <row r="682" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H682" s="10"/>
+      <c r="I682" s="8"/>
     </row>
     <row r="683" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H683" s="10"/>
+      <c r="I683" s="8"/>
     </row>
     <row r="684" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H684" s="10"/>
+      <c r="I684" s="8"/>
     </row>
     <row r="685" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H685" s="10"/>
+      <c r="I685" s="8"/>
     </row>
     <row r="686" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H686" s="10"/>
+      <c r="I686" s="8"/>
     </row>
     <row r="687" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H687" s="10"/>
+      <c r="I687" s="8"/>
     </row>
     <row r="688" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H688" s="10"/>
+      <c r="I688" s="8"/>
     </row>
     <row r="689" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H689" s="10"/>
+      <c r="I689" s="8"/>
     </row>
     <row r="690" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H690" s="10"/>
+      <c r="I690" s="8"/>
     </row>
     <row r="691" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H691" s="10"/>
+      <c r="I691" s="8"/>
     </row>
     <row r="692" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H692" s="10"/>
+      <c r="I692" s="8"/>
     </row>
     <row r="693" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H693" s="10"/>
+      <c r="I693" s="8"/>
     </row>
     <row r="694" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H694" s="10"/>
+      <c r="I694" s="8"/>
     </row>
     <row r="695" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H695" s="10"/>
+      <c r="I695" s="8"/>
     </row>
     <row r="696" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H696" s="10"/>
+      <c r="I696" s="8"/>
     </row>
     <row r="697" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H697" s="10"/>
+      <c r="I697" s="8"/>
     </row>
     <row r="698" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H698" s="10"/>
+      <c r="I698" s="8"/>
     </row>
     <row r="699" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H699" s="10"/>
+      <c r="I699" s="8"/>
     </row>
     <row r="700" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H700" s="10"/>
+      <c r="I700" s="8"/>
     </row>
     <row r="701" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H701" s="10"/>
+      <c r="I701" s="8"/>
     </row>
     <row r="702" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H702" s="10"/>
+      <c r="I702" s="8"/>
     </row>
     <row r="703" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H703" s="10"/>
+      <c r="I703" s="8"/>
     </row>
     <row r="704" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H704" s="10"/>
+      <c r="I704" s="8"/>
     </row>
     <row r="705" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H705" s="10"/>
+      <c r="I705" s="8"/>
     </row>
     <row r="706" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H706" s="10"/>
+      <c r="I706" s="8"/>
     </row>
     <row r="707" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H707" s="10"/>
+      <c r="I707" s="8"/>
     </row>
     <row r="708" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H708" s="10"/>
+      <c r="I708" s="8"/>
     </row>
     <row r="709" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H709" s="10"/>
+      <c r="I709" s="8"/>
     </row>
     <row r="710" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H710" s="10"/>
+      <c r="I710" s="8"/>
     </row>
     <row r="711" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H711" s="10"/>
+      <c r="I711" s="8"/>
     </row>
     <row r="712" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H712" s="10"/>
+      <c r="I712" s="8"/>
     </row>
     <row r="713" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H713" s="10"/>
+      <c r="I713" s="8"/>
     </row>
     <row r="714" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H714" s="10"/>
+      <c r="I714" s="8"/>
     </row>
     <row r="715" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H715" s="10"/>
+      <c r="I715" s="8"/>
     </row>
     <row r="716" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H716" s="10"/>
+      <c r="I716" s="8"/>
     </row>
     <row r="717" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H717" s="10"/>
+      <c r="I717" s="8"/>
     </row>
     <row r="718" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H718" s="10"/>
+      <c r="I718" s="8"/>
     </row>
     <row r="719" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H719" s="10"/>
+      <c r="I719" s="8"/>
     </row>
     <row r="720" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H720" s="10"/>
+      <c r="I720" s="8"/>
     </row>
     <row r="721" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H721" s="10"/>
+      <c r="I721" s="8"/>
     </row>
     <row r="722" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H722" s="10"/>
+      <c r="I722" s="8"/>
     </row>
     <row r="723" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H723" s="10"/>
+      <c r="I723" s="8"/>
     </row>
     <row r="724" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H724" s="10"/>
+      <c r="I724" s="8"/>
     </row>
     <row r="725" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H725" s="10"/>
+      <c r="I725" s="8"/>
     </row>
     <row r="726" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H726" s="10"/>
+      <c r="I726" s="8"/>
     </row>
     <row r="727" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H727" s="10"/>
+      <c r="I727" s="8"/>
     </row>
     <row r="728" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H728" s="10"/>
+      <c r="I728" s="8"/>
     </row>
     <row r="729" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H729" s="10"/>
+      <c r="I729" s="8"/>
     </row>
     <row r="730" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H730" s="10"/>
+      <c r="I730" s="8"/>
     </row>
     <row r="731" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H731" s="10"/>
+      <c r="I731" s="8"/>
     </row>
     <row r="732" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H732" s="10"/>
+      <c r="I732" s="8"/>
     </row>
     <row r="733" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H733" s="10"/>
+      <c r="I733" s="8"/>
     </row>
     <row r="734" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H734" s="10"/>
+      <c r="I734" s="8"/>
     </row>
     <row r="735" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H735" s="10"/>
+      <c r="I735" s="8"/>
     </row>
     <row r="736" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H736" s="10"/>
+      <c r="I736" s="8"/>
     </row>
     <row r="737" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H737" s="10"/>
+      <c r="I737" s="8"/>
     </row>
     <row r="738" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H738" s="10"/>
+      <c r="I738" s="8"/>
     </row>
     <row r="739" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H739" s="10"/>
+      <c r="I739" s="8"/>
     </row>
     <row r="740" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H740" s="10"/>
+      <c r="I740" s="8"/>
     </row>
     <row r="741" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H741" s="10"/>
+      <c r="I741" s="8"/>
     </row>
     <row r="742" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H742" s="10"/>
+      <c r="I742" s="8"/>
     </row>
     <row r="743" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H743" s="10"/>
+      <c r="I743" s="8"/>
     </row>
     <row r="744" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H744" s="10"/>
+      <c r="I744" s="8"/>
     </row>
     <row r="745" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H745" s="10"/>
+      <c r="I745" s="8"/>
     </row>
     <row r="746" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H746" s="10"/>
+      <c r="I746" s="8"/>
     </row>
     <row r="747" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H747" s="10"/>
+      <c r="I747" s="8"/>
     </row>
     <row r="748" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H748" s="10"/>
+      <c r="I748" s="8"/>
     </row>
     <row r="749" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H749" s="10"/>
+      <c r="I749" s="8"/>
     </row>
     <row r="750" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H750" s="10"/>
+      <c r="I750" s="8"/>
     </row>
     <row r="751" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H751" s="10"/>
+      <c r="I751" s="8"/>
     </row>
     <row r="752" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H752" s="10"/>
+      <c r="I752" s="8"/>
     </row>
     <row r="753" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H753" s="10"/>
+      <c r="I753" s="8"/>
     </row>
     <row r="754" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H754" s="10"/>
+      <c r="I754" s="8"/>
     </row>
     <row r="755" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H755" s="10"/>
+      <c r="I755" s="8"/>
     </row>
     <row r="756" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H756" s="10"/>
+      <c r="I756" s="8"/>
     </row>
     <row r="757" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H757" s="10"/>
+      <c r="I757" s="8"/>
     </row>
     <row r="758" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H758" s="10"/>
+      <c r="I758" s="8"/>
     </row>
     <row r="759" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H759" s="10"/>
+      <c r="I759" s="8"/>
     </row>
     <row r="760" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H760" s="10"/>
+      <c r="I760" s="8"/>
     </row>
     <row r="761" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H761" s="10"/>
+      <c r="I761" s="8"/>
     </row>
     <row r="762" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H762" s="10"/>
+      <c r="I762" s="8"/>
     </row>
     <row r="763" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H763" s="10"/>
+      <c r="I763" s="8"/>
     </row>
     <row r="764" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H764" s="10"/>
+      <c r="I764" s="8"/>
     </row>
     <row r="765" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H765" s="10"/>
+      <c r="I765" s="8"/>
     </row>
     <row r="766" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H766" s="10"/>
+      <c r="I766" s="8"/>
     </row>
     <row r="767" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H767" s="10"/>
+      <c r="I767" s="8"/>
     </row>
     <row r="768" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H768" s="10"/>
+      <c r="I768" s="8"/>
     </row>
     <row r="769" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H769" s="10"/>
+      <c r="I769" s="8"/>
     </row>
     <row r="770" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H770" s="10"/>
+      <c r="I770" s="8"/>
     </row>
     <row r="771" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H771" s="10"/>
+      <c r="I771" s="8"/>
     </row>
     <row r="772" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H772" s="10"/>
+      <c r="I772" s="8"/>
     </row>
     <row r="773" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H773" s="10"/>
+      <c r="I773" s="8"/>
     </row>
     <row r="774" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H774" s="10"/>
+      <c r="I774" s="8"/>
     </row>
     <row r="775" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H775" s="10"/>
+      <c r="I775" s="8"/>
     </row>
     <row r="776" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H776" s="10"/>
+      <c r="I776" s="8"/>
     </row>
     <row r="777" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H777" s="10"/>
+      <c r="I777" s="8"/>
     </row>
     <row r="778" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H778" s="10"/>
+      <c r="I778" s="8"/>
     </row>
     <row r="779" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H779" s="10"/>
+      <c r="I779" s="8"/>
     </row>
     <row r="780" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H780" s="10"/>
+      <c r="I780" s="8"/>
     </row>
     <row r="781" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H781" s="10"/>
+      <c r="I781" s="8"/>
     </row>
     <row r="782" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H782" s="10"/>
+      <c r="I782" s="8"/>
     </row>
     <row r="783" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H783" s="10"/>
+      <c r="I783" s="8"/>
     </row>
     <row r="784" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H784" s="10"/>
+      <c r="I784" s="8"/>
     </row>
     <row r="785" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H785" s="10"/>
+      <c r="I785" s="8"/>
     </row>
     <row r="786" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H786" s="10"/>
+      <c r="I786" s="8"/>
     </row>
     <row r="787" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H787" s="10"/>
+      <c r="I787" s="8"/>
     </row>
     <row r="788" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H788" s="10"/>
+      <c r="I788" s="8"/>
     </row>
     <row r="789" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H789" s="10"/>
+      <c r="I789" s="8"/>
     </row>
     <row r="790" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H790" s="10"/>
+      <c r="I790" s="8"/>
     </row>
     <row r="791" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H791" s="10"/>
+      <c r="I791" s="8"/>
     </row>
     <row r="792" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H792" s="10"/>
+      <c r="I792" s="8"/>
     </row>
     <row r="793" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H793" s="10"/>
+      <c r="I793" s="8"/>
     </row>
     <row r="794" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H794" s="10"/>
+      <c r="I794" s="8"/>
     </row>
     <row r="795" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H795" s="10"/>
+      <c r="I795" s="8"/>
     </row>
     <row r="796" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H796" s="10"/>
+      <c r="I796" s="8"/>
     </row>
     <row r="797" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H797" s="10"/>
+      <c r="I797" s="8"/>
     </row>
     <row r="798" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H798" s="10"/>
+      <c r="I798" s="8"/>
     </row>
     <row r="799" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H799" s="10"/>
+      <c r="I799" s="8"/>
     </row>
     <row r="800" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H800" s="10"/>
+      <c r="I800" s="8"/>
     </row>
     <row r="801" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H801" s="10"/>
+      <c r="I801" s="8"/>
     </row>
     <row r="802" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H802" s="10"/>
+      <c r="I802" s="8"/>
     </row>
     <row r="803" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H803" s="10"/>
+      <c r="I803" s="8"/>
     </row>
     <row r="804" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H804" s="10"/>
+      <c r="I804" s="8"/>
     </row>
     <row r="805" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H805" s="10"/>
+      <c r="I805" s="8"/>
     </row>
     <row r="806" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H806" s="10"/>
+      <c r="I806" s="8"/>
     </row>
     <row r="807" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H807" s="10"/>
+      <c r="I807" s="8"/>
     </row>
     <row r="808" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H808" s="10"/>
+      <c r="I808" s="8"/>
     </row>
     <row r="809" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H809" s="10"/>
+      <c r="I809" s="8"/>
     </row>
     <row r="810" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H810" s="10"/>
+      <c r="I810" s="8"/>
     </row>
     <row r="811" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H811" s="10"/>
+      <c r="I811" s="8"/>
     </row>
     <row r="812" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H812" s="10"/>
+      <c r="I812" s="8"/>
     </row>
     <row r="813" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H813" s="10"/>
+      <c r="I813" s="8"/>
     </row>
     <row r="814" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H814" s="10"/>
+      <c r="I814" s="8"/>
     </row>
     <row r="815" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H815" s="10"/>
+      <c r="I815" s="8"/>
     </row>
     <row r="816" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H816" s="10"/>
+      <c r="I816" s="8"/>
     </row>
     <row r="817" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H817" s="10"/>
+      <c r="I817" s="8"/>
     </row>
     <row r="818" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H818" s="10"/>
+      <c r="I818" s="8"/>
     </row>
     <row r="819" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H819" s="10"/>
+      <c r="I819" s="8"/>
     </row>
     <row r="820" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H820" s="10"/>
+      <c r="I820" s="8"/>
     </row>
     <row r="821" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H821" s="10"/>
+      <c r="I821" s="8"/>
     </row>
     <row r="822" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H822" s="10"/>
+      <c r="I822" s="8"/>
     </row>
     <row r="823" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H823" s="10"/>
+      <c r="I823" s="8"/>
     </row>
     <row r="824" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H824" s="10"/>
+      <c r="I824" s="8"/>
     </row>
     <row r="825" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H825" s="10"/>
+      <c r="I825" s="8"/>
     </row>
     <row r="826" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H826" s="10"/>
+      <c r="I826" s="8"/>
     </row>
     <row r="827" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H827" s="10"/>
+      <c r="I827" s="8"/>
     </row>
     <row r="828" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H828" s="10"/>
+      <c r="I828" s="8"/>
     </row>
     <row r="829" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H829" s="10"/>
+      <c r="I829" s="8"/>
     </row>
     <row r="830" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H830" s="10"/>
+      <c r="I830" s="8"/>
     </row>
     <row r="831" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H831" s="10"/>
+      <c r="I831" s="8"/>
     </row>
     <row r="832" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H832" s="10"/>
+      <c r="I832" s="8"/>
     </row>
     <row r="833" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H833" s="10"/>
+      <c r="I833" s="8"/>
     </row>
     <row r="834" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H834" s="10"/>
+      <c r="I834" s="8"/>
     </row>
     <row r="835" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H835" s="10"/>
+      <c r="I835" s="8"/>
     </row>
     <row r="836" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H836" s="10"/>
+      <c r="I836" s="8"/>
     </row>
     <row r="837" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H837" s="10"/>
+      <c r="I837" s="8"/>
     </row>
     <row r="838" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H838" s="10"/>
+      <c r="I838" s="8"/>
     </row>
     <row r="839" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H839" s="10"/>
+      <c r="I839" s="8"/>
     </row>
     <row r="840" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H840" s="10"/>
+      <c r="I840" s="8"/>
     </row>
     <row r="841" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H841" s="10"/>
+      <c r="I841" s="8"/>
     </row>
     <row r="842" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H842" s="10"/>
+      <c r="I842" s="8"/>
     </row>
     <row r="843" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H843" s="10"/>
+      <c r="I843" s="8"/>
     </row>
     <row r="844" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H844" s="10"/>
+      <c r="I844" s="8"/>
     </row>
     <row r="845" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H845" s="10"/>
+      <c r="I845" s="8"/>
     </row>
     <row r="846" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H846" s="10"/>
+      <c r="I846" s="8"/>
     </row>
     <row r="847" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H847" s="10"/>
+      <c r="I847" s="8"/>
     </row>
     <row r="848" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H848" s="10"/>
+      <c r="I848" s="8"/>
     </row>
     <row r="849" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H849" s="10"/>
+      <c r="I849" s="8"/>
     </row>
     <row r="850" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H850" s="10"/>
+      <c r="I850" s="8"/>
     </row>
     <row r="851" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H851" s="10"/>
+      <c r="I851" s="8"/>
     </row>
     <row r="852" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H852" s="10"/>
+      <c r="I852" s="8"/>
     </row>
     <row r="853" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H853" s="10"/>
+      <c r="I853" s="8"/>
     </row>
     <row r="854" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H854" s="10"/>
+      <c r="I854" s="8"/>
     </row>
     <row r="855" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H855" s="10"/>
+      <c r="I855" s="8"/>
     </row>
     <row r="856" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H856" s="10"/>
+      <c r="I856" s="8"/>
     </row>
     <row r="857" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H857" s="10"/>
+      <c r="I857" s="8"/>
     </row>
     <row r="858" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H858" s="10"/>
+      <c r="I858" s="8"/>
     </row>
     <row r="859" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H859" s="10"/>
+      <c r="I859" s="8"/>
     </row>
     <row r="860" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H860" s="10"/>
+      <c r="I860" s="8"/>
     </row>
     <row r="861" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H861" s="10"/>
+      <c r="I861" s="8"/>
     </row>
     <row r="862" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H862" s="10"/>
+      <c r="I862" s="8"/>
     </row>
     <row r="863" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H863" s="10"/>
+      <c r="I863" s="8"/>
     </row>
     <row r="864" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H864" s="10"/>
+      <c r="I864" s="8"/>
     </row>
     <row r="865" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H865" s="10"/>
+      <c r="I865" s="8"/>
     </row>
     <row r="866" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H866" s="10"/>
+      <c r="I866" s="8"/>
     </row>
     <row r="867" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H867" s="10"/>
+      <c r="I867" s="8"/>
     </row>
     <row r="868" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H868" s="10"/>
+      <c r="I868" s="8"/>
     </row>
     <row r="869" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H869" s="10"/>
+      <c r="I869" s="8"/>
     </row>
     <row r="870" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H870" s="10"/>
+      <c r="I870" s="8"/>
     </row>
     <row r="871" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H871" s="10"/>
+      <c r="I871" s="8"/>
     </row>
     <row r="872" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H872" s="10"/>
+      <c r="I872" s="8"/>
     </row>
     <row r="873" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H873" s="10"/>
+      <c r="I873" s="8"/>
     </row>
     <row r="874" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H874" s="10"/>
+      <c r="I874" s="8"/>
     </row>
     <row r="875" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H875" s="10"/>
+      <c r="I875" s="8"/>
     </row>
     <row r="876" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H876" s="10"/>
+      <c r="I876" s="8"/>
     </row>
     <row r="877" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H877" s="10"/>
+      <c r="I877" s="8"/>
     </row>
     <row r="878" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H878" s="10"/>
+      <c r="I878" s="8"/>
     </row>
     <row r="879" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H879" s="10"/>
+      <c r="I879" s="8"/>
     </row>
     <row r="880" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H880" s="10"/>
+      <c r="I880" s="8"/>
     </row>
     <row r="881" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H881" s="10"/>
+      <c r="I881" s="8"/>
     </row>
     <row r="882" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H882" s="10"/>
+      <c r="I882" s="8"/>
     </row>
     <row r="883" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H883" s="10"/>
+      <c r="I883" s="8"/>
     </row>
     <row r="884" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H884" s="10"/>
+      <c r="I884" s="8"/>
     </row>
     <row r="885" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H885" s="10"/>
+      <c r="I885" s="8"/>
     </row>
     <row r="886" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H886" s="10"/>
+      <c r="I886" s="8"/>
     </row>
     <row r="887" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H887" s="10"/>
+      <c r="I887" s="8"/>
     </row>
     <row r="888" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H888" s="10"/>
+      <c r="I888" s="8"/>
     </row>
     <row r="889" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H889" s="10"/>
+      <c r="I889" s="8"/>
     </row>
     <row r="890" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H890" s="10"/>
+      <c r="I890" s="8"/>
     </row>
     <row r="891" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H891" s="10"/>
+      <c r="I891" s="8"/>
     </row>
     <row r="892" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H892" s="10"/>
+      <c r="I892" s="8"/>
     </row>
     <row r="893" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H893" s="10"/>
+      <c r="I893" s="8"/>
     </row>
     <row r="894" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H894" s="10"/>
+      <c r="I894" s="8"/>
     </row>
     <row r="895" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H895" s="10"/>
+      <c r="I895" s="8"/>
     </row>
     <row r="896" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H896" s="10"/>
+      <c r="I896" s="8"/>
     </row>
     <row r="897" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H897" s="10"/>
+      <c r="I897" s="8"/>
     </row>
     <row r="898" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H898" s="10"/>
+      <c r="I898" s="8"/>
     </row>
     <row r="899" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H899" s="10"/>
+      <c r="I899" s="8"/>
     </row>
     <row r="900" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H900" s="10"/>
+      <c r="I900" s="8"/>
     </row>
     <row r="901" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H901" s="10"/>
+      <c r="I901" s="8"/>
     </row>
     <row r="902" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H902" s="10"/>
+      <c r="I902" s="8"/>
     </row>
     <row r="903" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H903" s="10"/>
+      <c r="I903" s="8"/>
     </row>
     <row r="904" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H904" s="10"/>
+      <c r="I904" s="8"/>
     </row>
     <row r="905" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H905" s="10"/>
+      <c r="I905" s="8"/>
     </row>
     <row r="906" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H906" s="10"/>
+      <c r="I906" s="8"/>
     </row>
     <row r="907" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H907" s="10"/>
+      <c r="I907" s="8"/>
     </row>
     <row r="908" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H908" s="10"/>
+      <c r="I908" s="8"/>
     </row>
     <row r="909" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H909" s="10"/>
+      <c r="I909" s="8"/>
     </row>
     <row r="910" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H910" s="10"/>
+      <c r="I910" s="8"/>
     </row>
     <row r="911" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H911" s="10"/>
+      <c r="I911" s="8"/>
     </row>
     <row r="912" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H912" s="10"/>
+      <c r="I912" s="8"/>
     </row>
     <row r="913" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H913" s="10"/>
+      <c r="I913" s="8"/>
     </row>
     <row r="914" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H914" s="10"/>
+      <c r="I914" s="8"/>
     </row>
     <row r="915" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H915" s="10"/>
+      <c r="I915" s="8"/>
     </row>
     <row r="916" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H916" s="10"/>
+      <c r="I916" s="8"/>
     </row>
     <row r="917" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H917" s="10"/>
+      <c r="I917" s="8"/>
     </row>
     <row r="918" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H918" s="10"/>
+      <c r="I918" s="8"/>
     </row>
     <row r="919" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H919" s="10"/>
+      <c r="I919" s="8"/>
     </row>
     <row r="920" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H920" s="10"/>
+      <c r="I920" s="8"/>
     </row>
     <row r="921" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H921" s="10"/>
+      <c r="I921" s="8"/>
     </row>
     <row r="922" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H922" s="10"/>
+      <c r="I922" s="8"/>
     </row>
     <row r="923" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H923" s="10"/>
+      <c r="I923" s="8"/>
     </row>
     <row r="924" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H924" s="10"/>
+      <c r="I924" s="8"/>
     </row>
     <row r="925" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H925" s="10"/>
+      <c r="I925" s="8"/>
     </row>
     <row r="926" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H926" s="10"/>
+      <c r="I926" s="8"/>
     </row>
     <row r="927" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H927" s="10"/>
+      <c r="I927" s="8"/>
     </row>
     <row r="928" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H928" s="10"/>
+      <c r="I928" s="8"/>
     </row>
     <row r="929" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H929" s="10"/>
+      <c r="I929" s="8"/>
     </row>
     <row r="930" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H930" s="10"/>
+      <c r="I930" s="8"/>
     </row>
     <row r="931" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H931" s="10"/>
+      <c r="I931" s="8"/>
     </row>
     <row r="932" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H932" s="10"/>
+      <c r="I932" s="8"/>
     </row>
     <row r="933" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H933" s="10"/>
+      <c r="I933" s="8"/>
     </row>
     <row r="934" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H934" s="10"/>
+      <c r="I934" s="8"/>
     </row>
     <row r="935" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H935" s="10"/>
+      <c r="I935" s="8"/>
     </row>
     <row r="936" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H936" s="10"/>
+      <c r="I936" s="8"/>
     </row>
     <row r="937" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H937" s="10"/>
+      <c r="I937" s="8"/>
     </row>
     <row r="938" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H938" s="10"/>
+      <c r="I938" s="8"/>
     </row>
     <row r="939" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H939" s="10"/>
+      <c r="I939" s="8"/>
     </row>
     <row r="940" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H940" s="10"/>
+      <c r="I940" s="8"/>
     </row>
     <row r="941" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H941" s="10"/>
+      <c r="I941" s="8"/>
     </row>
     <row r="942" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H942" s="10"/>
+      <c r="I942" s="8"/>
     </row>
     <row r="943" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H943" s="10"/>
+      <c r="I943" s="8"/>
     </row>
     <row r="944" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H944" s="10"/>
+      <c r="I944" s="8"/>
     </row>
     <row r="945" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H945" s="10"/>
+      <c r="I945" s="8"/>
     </row>
     <row r="946" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H946" s="10"/>
+      <c r="I946" s="8"/>
     </row>
     <row r="947" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H947" s="10"/>
+      <c r="I947" s="8"/>
     </row>
     <row r="948" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H948" s="10"/>
+      <c r="I948" s="8"/>
     </row>
     <row r="949" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H949" s="10"/>
+      <c r="I949" s="8"/>
     </row>
     <row r="950" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H950" s="10"/>
+      <c r="I950" s="8"/>
     </row>
     <row r="951" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H951" s="10"/>
+      <c r="I951" s="8"/>
     </row>
     <row r="952" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H952" s="10"/>
+      <c r="I952" s="8"/>
     </row>
     <row r="953" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H953" s="10"/>
+      <c r="I953" s="8"/>
     </row>
     <row r="954" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H954" s="10"/>
+      <c r="I954" s="8"/>
     </row>
     <row r="955" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H955" s="10"/>
+      <c r="I955" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Alphabet Learning Resources: from json to sql
</commit_message>
<xml_diff>
--- a/data/master_sheets.xlsx
+++ b/data/master_sheets.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2309" uniqueCount="800">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="803">
   <si>
     <t xml:space="preserve">Georgian</t>
   </si>
@@ -2403,7 +2403,7 @@
     <t xml:space="preserve">Alphabet</t>
   </si>
   <si>
-    <t xml:space="preserve">vowels</t>
+    <t xml:space="preserve">Vowels</t>
   </si>
   <si>
     <t xml:space="preserve">monologue</t>
@@ -2412,7 +2412,16 @@
     <t xml:space="preserve">უ </t>
   </si>
   <si>
-    <t xml:space="preserve">consonants</t>
+    <t xml:space="preserve">Letters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ejectives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affricates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gutturals</t>
   </si>
   <si>
     <t xml:space="preserve">Basic Survival</t>
@@ -2657,7 +2666,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P155"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.23"/>
   </cols>
@@ -9052,7 +9061,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H51"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.5"/>
   </cols>
@@ -10099,12 +10108,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1012"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I1059"/>
+  <sheetFormatPr defaultColWidth="12.6953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="10.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="9.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20.76"/>
   </cols>
@@ -10308,1312 +10317,1318 @@
         <v>792</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>796</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="I8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>323</v>
+        <v>25</v>
       </c>
       <c r="I9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>331</v>
+        <v>30</v>
       </c>
       <c r="I10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>336</v>
+        <v>34</v>
       </c>
       <c r="I11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>342</v>
+        <v>38</v>
       </c>
       <c r="I12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>746</v>
+        <v>42</v>
       </c>
       <c r="I13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>349</v>
+        <v>46</v>
       </c>
       <c r="I14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>360</v>
+        <v>50</v>
       </c>
       <c r="I15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>371</v>
+        <v>54</v>
       </c>
       <c r="I16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>368</v>
+        <v>58</v>
       </c>
       <c r="I17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>731</v>
+        <v>62</v>
       </c>
       <c r="I18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E19" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>378</v>
+        <v>66</v>
       </c>
       <c r="I19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E20" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>384</v>
+        <v>70</v>
       </c>
       <c r="I20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>388</v>
+        <v>74</v>
       </c>
       <c r="I21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>400</v>
+        <v>78</v>
       </c>
       <c r="I22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>742</v>
+        <v>82</v>
       </c>
       <c r="I23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>4</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>405</v>
+        <v>86</v>
       </c>
       <c r="I24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E25" s="5" t="n">
         <v>4</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>411</v>
+        <v>90</v>
       </c>
       <c r="I25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>326</v>
+        <v>2</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E26" s="5" t="n">
         <v>4</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>746</v>
+        <v>94</v>
       </c>
       <c r="I26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>418</v>
+      <c r="D27" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>415</v>
+        <v>98</v>
       </c>
       <c r="I27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>418</v>
+      <c r="D28" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>424</v>
+        <v>102</v>
       </c>
       <c r="I28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>418</v>
+      <c r="D29" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>433</v>
+        <v>106</v>
       </c>
       <c r="I29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>418</v>
+      <c r="D30" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>750</v>
+        <v>110</v>
       </c>
       <c r="I30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D31" s="5" t="s">
-        <v>418</v>
+      <c r="D31" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>436</v>
+        <v>114</v>
       </c>
       <c r="I31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>418</v>
+      <c r="D32" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>444</v>
+        <v>118</v>
       </c>
       <c r="I32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>418</v>
+      <c r="D33" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>441</v>
+        <v>122</v>
       </c>
       <c r="I33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>418</v>
+      <c r="D34" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E34" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F34" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F34" s="5" t="n">
-        <v>4</v>
-      </c>
       <c r="G34" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>754</v>
+        <v>126</v>
       </c>
       <c r="I34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C35" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>418</v>
+      <c r="D35" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E35" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F35" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="F35" s="5" t="n">
-        <v>1</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>452</v>
+        <v>130</v>
       </c>
       <c r="I35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>418</v>
+      <c r="D36" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>448</v>
+        <v>134</v>
       </c>
       <c r="I36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>418</v>
+      <c r="D37" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>454</v>
+        <v>138</v>
       </c>
       <c r="I37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C38" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="5" t="s">
-        <v>418</v>
+      <c r="D38" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>464</v>
+        <v>142</v>
       </c>
       <c r="I38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C39" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D39" s="5" t="s">
-        <v>418</v>
+      <c r="D39" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E39" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F39" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F39" s="5" t="n">
-        <v>5</v>
-      </c>
       <c r="G39" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>754</v>
+        <v>146</v>
       </c>
       <c r="I39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>472</v>
+        <v>2</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>796</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>520</v>
+        <v>150</v>
       </c>
       <c r="I40" s="9"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C41" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D41" s="5" t="s">
-        <v>472</v>
+      <c r="D41" s="4" t="s">
+        <v>797</v>
       </c>
       <c r="E41" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>528</v>
+        <v>94</v>
       </c>
       <c r="I41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C42" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D42" s="5" t="s">
-        <v>472</v>
+      <c r="D42" s="4" t="s">
+        <v>797</v>
       </c>
       <c r="E42" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>534</v>
+        <v>78</v>
       </c>
       <c r="I42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C43" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>472</v>
+      <c r="D43" s="4" t="s">
+        <v>797</v>
       </c>
       <c r="E43" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>799</v>
+        <v>58</v>
       </c>
       <c r="I43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C44" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>472</v>
+      <c r="D44" s="4" t="s">
+        <v>797</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>510</v>
+        <v>134</v>
       </c>
       <c r="I44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C45" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D45" s="5" t="s">
-        <v>472</v>
+      <c r="D45" s="4" t="s">
+        <v>797</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>515</v>
+        <v>138</v>
       </c>
       <c r="I45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C46" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D46" s="5" t="s">
-        <v>472</v>
+      <c r="D46" s="4" t="s">
+        <v>797</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>500</v>
+        <v>114</v>
       </c>
       <c r="I46" s="9"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>472</v>
+        <v>4</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>798</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>505</v>
+        <v>126</v>
       </c>
       <c r="I47" s="9"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>472</v>
+        <v>4</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>798</v>
       </c>
       <c r="E48" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F48" s="5" t="n">
-        <v>5</v>
-      </c>
       <c r="G48" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>766</v>
+        <v>130</v>
       </c>
       <c r="I48" s="9"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C49" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>798</v>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>472</v>
-      </c>
-      <c r="E49" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F49" s="5" t="n">
-        <v>1</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>483</v>
+        <v>122</v>
       </c>
       <c r="I49" s="9"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C50" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>472</v>
+        <v>4</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>798</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G50" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>469</v>
+        <v>146</v>
       </c>
       <c r="I50" s="9"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>472</v>
+        <v>4</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>798</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>479</v>
+        <v>134</v>
       </c>
       <c r="I51" s="9"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C52" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>472</v>
+        <v>4</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>798</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G52" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>485</v>
+        <v>138</v>
       </c>
       <c r="I52" s="9"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C53" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>472</v>
+        <v>5</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>799</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>489</v>
+        <v>142</v>
       </c>
       <c r="I53" s="9"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C54" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>472</v>
+        <v>5</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>799</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G54" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>495</v>
+        <v>110</v>
       </c>
       <c r="I54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C55" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>799</v>
+      </c>
+      <c r="E55" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D55" s="5" t="s">
-        <v>472</v>
-      </c>
-      <c r="E55" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F55" s="5" t="n">
-        <v>7</v>
-      </c>
       <c r="G55" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>759</v>
+        <v>114</v>
       </c>
       <c r="I55" s="9"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="C56" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>472</v>
+        <v>5</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>799</v>
       </c>
       <c r="E56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="F56" s="5" t="n">
-        <v>1</v>
       </c>
       <c r="G56" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>539</v>
+        <v>106</v>
       </c>
       <c r="I56" s="9"/>
     </row>
@@ -11622,16 +11637,16 @@
         <v>1</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C57" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>472</v>
+        <v>326</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F57" s="5" t="n">
         <v>2</v>
@@ -11640,24 +11655,25 @@
         <v>794</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>544</v>
-      </c>
+        <v>331</v>
+      </c>
+      <c r="I57" s="9"/>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C58" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>472</v>
+        <v>326</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F58" s="5" t="n">
         <v>3</v>
@@ -11666,24 +11682,25 @@
         <v>794</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>548</v>
-      </c>
+        <v>336</v>
+      </c>
+      <c r="I58" s="9"/>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>472</v>
+        <v>326</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F59" s="5" t="n">
         <v>4</v>
@@ -11692,50 +11709,52 @@
         <v>794</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>582</v>
-      </c>
+        <v>342</v>
+      </c>
+      <c r="I59" s="9"/>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C60" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>472</v>
+        <v>326</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F60" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>759</v>
-      </c>
+        <v>746</v>
+      </c>
+      <c r="I60" s="9"/>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C61" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="5" t="n">
         <v>1</v>
@@ -11744,24 +11763,25 @@
         <v>794</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>637</v>
-      </c>
+        <v>349</v>
+      </c>
+      <c r="I61" s="9"/>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C62" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" s="5" t="n">
         <v>2</v>
@@ -11770,24 +11790,25 @@
         <v>794</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>644</v>
-      </c>
+        <v>360</v>
+      </c>
+      <c r="I62" s="9"/>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C63" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="5" t="n">
         <v>3</v>
@@ -11796,24 +11817,25 @@
         <v>794</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>648</v>
-      </c>
+        <v>371</v>
+      </c>
+      <c r="I63" s="9"/>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C64" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F64" s="5" t="n">
         <v>4</v>
@@ -11822,463 +11844,481 @@
         <v>794</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>652</v>
-      </c>
+        <v>368</v>
+      </c>
+      <c r="I64" s="9"/>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F65" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>656</v>
-      </c>
+        <v>731</v>
+      </c>
+      <c r="I65" s="9"/>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C66" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G66" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>660</v>
-      </c>
+        <v>378</v>
+      </c>
+      <c r="I66" s="9"/>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C67" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G67" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H67" s="5" t="s">
-        <v>664</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="I67" s="9"/>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G68" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H68" s="5" t="s">
-        <v>668</v>
-      </c>
+        <v>388</v>
+      </c>
+      <c r="I68" s="9"/>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C69" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F69" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="D69" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="E69" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" s="5" t="n">
-        <v>9</v>
       </c>
       <c r="G69" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H69" s="5" t="s">
-        <v>672</v>
-      </c>
+        <v>400</v>
+      </c>
+      <c r="I69" s="9"/>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C70" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>640</v>
+        <v>326</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="H70" s="5" t="s">
-        <v>676</v>
-      </c>
+        <v>742</v>
+      </c>
+      <c r="I70" s="9"/>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C71" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="E71" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D71" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="E71" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="F71" s="5" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G71" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H71" s="5" t="s">
-        <v>680</v>
-      </c>
+        <v>405</v>
+      </c>
+      <c r="I71" s="9"/>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C72" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="E72" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D72" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="E72" s="5" t="n">
+      <c r="F72" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="F72" s="5" t="n">
-        <v>1</v>
       </c>
       <c r="G72" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>684</v>
-      </c>
+        <v>411</v>
+      </c>
+      <c r="I72" s="9"/>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C73" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="E73" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D73" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="E73" s="5" t="n">
-        <v>2</v>
-      </c>
       <c r="F73" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>688</v>
-      </c>
+        <v>746</v>
+      </c>
+      <c r="I73" s="9"/>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C74" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>640</v>
+        <v>418</v>
       </c>
       <c r="E74" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G74" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>692</v>
-      </c>
+        <v>415</v>
+      </c>
+      <c r="I74" s="9"/>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C75" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>640</v>
+        <v>418</v>
       </c>
       <c r="E75" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="F75" s="5" t="n">
-        <v>4</v>
       </c>
       <c r="G75" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H75" s="5" t="s">
-        <v>696</v>
-      </c>
+        <v>424</v>
+      </c>
+      <c r="I75" s="9"/>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C76" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>640</v>
+        <v>418</v>
       </c>
       <c r="E76" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G76" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>700</v>
-      </c>
+        <v>433</v>
+      </c>
+      <c r="I76" s="9"/>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C77" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="E77" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D77" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="E77" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F77" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="G77" s="5" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="H77" s="5" t="s">
-        <v>704</v>
-      </c>
+        <v>750</v>
+      </c>
+      <c r="I77" s="9"/>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C78" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>640</v>
+        <v>418</v>
       </c>
       <c r="E78" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F78" s="5" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G78" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H78" s="5" t="s">
-        <v>708</v>
-      </c>
+        <v>436</v>
+      </c>
+      <c r="I78" s="9"/>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C79" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>640</v>
+        <v>418</v>
       </c>
       <c r="E79" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F79" s="5" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G79" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H79" s="5" t="s">
-        <v>712</v>
-      </c>
+        <v>444</v>
+      </c>
+      <c r="I79" s="9"/>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C80" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>640</v>
+        <v>418</v>
       </c>
       <c r="E80" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F80" s="5" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G80" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H80" s="5" t="s">
-        <v>716</v>
-      </c>
+        <v>441</v>
+      </c>
+      <c r="I80" s="9"/>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C81" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>640</v>
+        <v>418</v>
       </c>
       <c r="E81" s="5" t="n">
         <v>2</v>
       </c>
       <c r="F81" s="5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="H81" s="5" t="s">
-        <v>720</v>
-      </c>
+        <v>754</v>
+      </c>
+      <c r="I81" s="9"/>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C82" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>551</v>
+        <v>418</v>
       </c>
       <c r="E82" s="5" t="n">
         <v>3</v>
@@ -12290,21 +12330,22 @@
         <v>794</v>
       </c>
       <c r="H82" s="5" t="s">
-        <v>559</v>
-      </c>
+        <v>452</v>
+      </c>
+      <c r="I82" s="9"/>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C83" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>551</v>
+        <v>418</v>
       </c>
       <c r="E83" s="5" t="n">
         <v>3</v>
@@ -12316,21 +12357,22 @@
         <v>794</v>
       </c>
       <c r="H83" s="5" t="s">
-        <v>564</v>
-      </c>
+        <v>448</v>
+      </c>
+      <c r="I83" s="9"/>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C84" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>551</v>
+        <v>418</v>
       </c>
       <c r="E84" s="5" t="n">
         <v>3</v>
@@ -12342,21 +12384,22 @@
         <v>794</v>
       </c>
       <c r="H84" s="5" t="s">
-        <v>568</v>
-      </c>
+        <v>454</v>
+      </c>
+      <c r="I84" s="9"/>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C85" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>551</v>
+        <v>418</v>
       </c>
       <c r="E85" s="5" t="n">
         <v>3</v>
@@ -12368,21 +12411,22 @@
         <v>794</v>
       </c>
       <c r="H85" s="5" t="s">
-        <v>572</v>
-      </c>
+        <v>464</v>
+      </c>
+      <c r="I85" s="9"/>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C86" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>551</v>
+        <v>418</v>
       </c>
       <c r="E86" s="5" t="n">
         <v>3</v>
@@ -12391,568 +12435,1667 @@
         <v>5</v>
       </c>
       <c r="G86" s="5" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>575</v>
-      </c>
+        <v>754</v>
+      </c>
+      <c r="I86" s="9"/>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C87" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>551</v>
+        <v>472</v>
       </c>
       <c r="E87" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F87" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G87" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H87" s="5" t="s">
-        <v>579</v>
-      </c>
+        <v>520</v>
+      </c>
+      <c r="I87" s="9"/>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C88" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>551</v>
+        <v>472</v>
       </c>
       <c r="E88" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F88" s="5" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G88" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H88" s="5" t="s">
-        <v>585</v>
-      </c>
+        <v>528</v>
+      </c>
+      <c r="I88" s="9"/>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C89" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>551</v>
+        <v>472</v>
       </c>
       <c r="E89" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="F89" s="5" t="n">
-        <v>8</v>
       </c>
       <c r="G89" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H89" s="5" t="s">
-        <v>582</v>
-      </c>
+        <v>534</v>
+      </c>
+      <c r="I89" s="9"/>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C90" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D90" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E90" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="D90" s="5" t="s">
-        <v>551</v>
-      </c>
-      <c r="E90" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F90" s="5" t="n">
-        <v>9</v>
       </c>
       <c r="G90" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H90" s="5" t="s">
-        <v>586</v>
-      </c>
+        <v>802</v>
+      </c>
+      <c r="I90" s="9"/>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C91" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>551</v>
+        <v>472</v>
       </c>
       <c r="E91" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F91" s="5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G91" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H91" s="5" t="s">
-        <v>770</v>
-      </c>
+        <v>510</v>
+      </c>
+      <c r="I91" s="9"/>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C92" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>599</v>
+        <v>472</v>
       </c>
       <c r="E92" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F92" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G92" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H92" s="5" t="s">
-        <v>596</v>
-      </c>
+        <v>515</v>
+      </c>
+      <c r="I92" s="9"/>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C93" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>599</v>
+        <v>472</v>
       </c>
       <c r="E93" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F93" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G93" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H93" s="5" t="s">
-        <v>605</v>
-      </c>
+        <v>500</v>
+      </c>
+      <c r="I93" s="9"/>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C94" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E94" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="D94" s="5" t="s">
-        <v>599</v>
-      </c>
-      <c r="E94" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F94" s="5" t="n">
-        <v>3</v>
       </c>
       <c r="G94" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H94" s="5" t="s">
-        <v>609</v>
-      </c>
+        <v>505</v>
+      </c>
+      <c r="I94" s="9"/>
     </row>
     <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C95" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>599</v>
+        <v>472</v>
       </c>
       <c r="E95" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F95" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G95" s="5" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="H95" s="5" t="s">
-        <v>613</v>
-      </c>
+        <v>766</v>
+      </c>
+      <c r="I95" s="9"/>
     </row>
     <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C96" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>599</v>
+        <v>472</v>
       </c>
       <c r="E96" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F96" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G96" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H96" s="5" t="s">
-        <v>616</v>
-      </c>
+        <v>483</v>
+      </c>
+      <c r="I96" s="9"/>
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C97" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>599</v>
+        <v>472</v>
       </c>
       <c r="E97" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F97" s="5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G97" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H97" s="5" t="s">
-        <v>620</v>
-      </c>
+        <v>469</v>
+      </c>
+      <c r="I97" s="9"/>
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C98" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>599</v>
+        <v>472</v>
       </c>
       <c r="E98" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F98" s="5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G98" s="5" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="H98" s="5" t="s">
-        <v>778</v>
-      </c>
+        <v>479</v>
+      </c>
+      <c r="I98" s="9"/>
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C99" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E99" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F99" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="D99" s="5" t="s">
-        <v>626</v>
-      </c>
-      <c r="E99" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F99" s="5" t="n">
-        <v>1</v>
       </c>
       <c r="G99" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H99" s="5" t="s">
-        <v>623</v>
-      </c>
+        <v>485</v>
+      </c>
+      <c r="I99" s="9"/>
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C100" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D100" s="5" t="s">
-        <v>626</v>
+        <v>472</v>
       </c>
       <c r="E100" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F100" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="F100" s="5" t="n">
-        <v>2</v>
       </c>
       <c r="G100" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H100" s="5" t="s">
-        <v>629</v>
-      </c>
+        <v>489</v>
+      </c>
+      <c r="I100" s="9"/>
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C101" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>626</v>
+        <v>472</v>
       </c>
       <c r="E101" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F101" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G101" s="5" t="s">
         <v>794</v>
       </c>
       <c r="H101" s="5" t="s">
-        <v>633</v>
-      </c>
+        <v>495</v>
+      </c>
+      <c r="I101" s="9"/>
     </row>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C102" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E102" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F102" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G102" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="H102" s="5" t="s">
+        <v>759</v>
+      </c>
+      <c r="I102" s="9"/>
+    </row>
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C103" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E103" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="F103" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H103" s="5" t="s">
+        <v>539</v>
+      </c>
+      <c r="I103" s="9"/>
+    </row>
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C104" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E104" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F104" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G104" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H104" s="5" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C105" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E105" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F105" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G105" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H105" s="5" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C106" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E106" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F106" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H106" s="5" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C107" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="E107" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G107" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="H107" s="5" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C108" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E108" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H108" s="5" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C109" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E109" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G109" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H109" s="5" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C110" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E110" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G110" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H110" s="5" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C111" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E111" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G111" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H111" s="5" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C112" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E112" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G112" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H112" s="5" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C113" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E113" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G113" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H113" s="5" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C114" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E114" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G114" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H114" s="5" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C115" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E115" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G115" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H115" s="5" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C116" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D116" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E116" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G116" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H116" s="5" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C117" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E117" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G117" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H117" s="5" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C118" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E118" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="G118" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H118" s="5" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C119" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E119" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F119" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G119" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H119" s="5" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C120" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E120" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F120" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G120" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H120" s="5" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C121" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E121" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F121" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G121" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H121" s="5" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C122" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E122" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F122" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G122" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H122" s="5" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C123" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E123" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F123" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G123" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H123" s="5" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C124" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F124" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G124" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H124" s="5" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C125" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E125" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F125" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G125" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H125" s="5" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C126" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E126" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F126" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G126" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H126" s="5" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C127" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E127" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F127" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G127" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H127" s="5" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C128" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="E128" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F128" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G128" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H128" s="5" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C129" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E129" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F129" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G129" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H129" s="5" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C130" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E130" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F130" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G130" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H130" s="5" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C131" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E131" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F131" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G131" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H131" s="5" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C132" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E132" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F132" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G132" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H132" s="5" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C133" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E133" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F133" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G133" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H133" s="5" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C134" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E134" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F134" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G134" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H134" s="5" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C135" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E135" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F135" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G135" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H135" s="5" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C136" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E136" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F136" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G136" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H136" s="5" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B137" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C137" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E137" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F137" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G137" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H137" s="5" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B138" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C138" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E138" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F138" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G138" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="H138" s="5" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B139" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C139" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="E139" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F139" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G139" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H139" s="5" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C140" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="E140" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F140" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G140" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H140" s="5" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C141" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="E141" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F141" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G141" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H141" s="5" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B142" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C142" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="E142" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F142" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G142" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H142" s="5" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B143" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C143" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="E143" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F143" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G143" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H143" s="5" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B144" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C144" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="E144" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F144" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G144" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H144" s="5" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C145" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="E145" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F145" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G145" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="H145" s="5" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B146" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C146" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D146" s="5" t="s">
         <v>626</v>
       </c>
-      <c r="E102" s="5" t="n">
+      <c r="E146" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F102" s="5" t="n">
+      <c r="F146" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G146" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H146" s="5" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B147" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C147" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="G102" s="5" t="s">
-        <v>798</v>
-      </c>
-      <c r="H102" s="5" t="s">
+      <c r="D147" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="E147" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F147" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G147" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H147" s="5" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B148" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C148" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D148" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="E148" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F148" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G148" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="H148" s="5" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B149" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C149" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D149" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="E149" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F149" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G149" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="H149" s="5" t="s">
         <v>781</v>
       </c>
-    </row>
-    <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I151" s="10"/>
-    </row>
-    <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I152" s="10"/>
-    </row>
-    <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I153" s="10"/>
-    </row>
-    <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I154" s="10"/>
-    </row>
-    <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I155" s="10"/>
-    </row>
-    <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I156" s="10"/>
-    </row>
-    <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I157" s="10"/>
-    </row>
-    <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I158" s="10"/>
-    </row>
-    <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I159" s="10"/>
-    </row>
-    <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I160" s="10"/>
-    </row>
-    <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I161" s="10"/>
-    </row>
-    <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I162" s="10"/>
-    </row>
-    <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I163" s="10"/>
-    </row>
-    <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I164" s="10"/>
-    </row>
-    <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I165" s="10"/>
-    </row>
-    <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I166" s="10"/>
-    </row>
-    <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I167" s="10"/>
-    </row>
-    <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I168" s="10"/>
-    </row>
-    <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I169" s="10"/>
-    </row>
-    <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I170" s="10"/>
-    </row>
-    <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I171" s="10"/>
-    </row>
-    <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I172" s="10"/>
-    </row>
-    <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I173" s="10"/>
-    </row>
-    <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I174" s="10"/>
-    </row>
-    <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I175" s="10"/>
-    </row>
-    <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I176" s="10"/>
-    </row>
-    <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I177" s="10"/>
-    </row>
-    <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I178" s="10"/>
-    </row>
-    <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I179" s="10"/>
-    </row>
-    <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I180" s="10"/>
-    </row>
-    <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I181" s="10"/>
-    </row>
-    <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I182" s="10"/>
-    </row>
-    <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I183" s="10"/>
-    </row>
-    <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I184" s="10"/>
-    </row>
-    <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I185" s="10"/>
-    </row>
-    <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I186" s="10"/>
-    </row>
-    <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I187" s="10"/>
-    </row>
-    <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I188" s="10"/>
-    </row>
-    <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I189" s="10"/>
-    </row>
-    <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I190" s="10"/>
-    </row>
-    <row r="191" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I191" s="10"/>
-    </row>
-    <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I192" s="10"/>
-    </row>
-    <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I193" s="10"/>
-    </row>
-    <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I194" s="10"/>
-    </row>
-    <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I195" s="10"/>
-    </row>
-    <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I196" s="10"/>
-    </row>
-    <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I197" s="10"/>
     </row>
     <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I198" s="10"/>
@@ -15398,6 +16541,147 @@
     </row>
     <row r="1012" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I1012" s="10"/>
+    </row>
+    <row r="1013" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1013" s="10"/>
+    </row>
+    <row r="1014" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1014" s="10"/>
+    </row>
+    <row r="1015" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1015" s="10"/>
+    </row>
+    <row r="1016" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1016" s="10"/>
+    </row>
+    <row r="1017" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1017" s="10"/>
+    </row>
+    <row r="1018" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1018" s="10"/>
+    </row>
+    <row r="1019" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1019" s="10"/>
+    </row>
+    <row r="1020" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1020" s="10"/>
+    </row>
+    <row r="1021" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1021" s="10"/>
+    </row>
+    <row r="1022" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1022" s="10"/>
+    </row>
+    <row r="1023" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1023" s="10"/>
+    </row>
+    <row r="1024" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1024" s="10"/>
+    </row>
+    <row r="1025" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1025" s="10"/>
+    </row>
+    <row r="1026" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1026" s="10"/>
+    </row>
+    <row r="1027" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1027" s="10"/>
+    </row>
+    <row r="1028" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1028" s="10"/>
+    </row>
+    <row r="1029" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1029" s="10"/>
+    </row>
+    <row r="1030" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1030" s="10"/>
+    </row>
+    <row r="1031" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1031" s="10"/>
+    </row>
+    <row r="1032" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1032" s="10"/>
+    </row>
+    <row r="1033" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1033" s="10"/>
+    </row>
+    <row r="1034" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1034" s="10"/>
+    </row>
+    <row r="1035" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1035" s="10"/>
+    </row>
+    <row r="1036" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1036" s="10"/>
+    </row>
+    <row r="1037" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1037" s="10"/>
+    </row>
+    <row r="1038" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1038" s="10"/>
+    </row>
+    <row r="1039" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1039" s="10"/>
+    </row>
+    <row r="1040" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1040" s="10"/>
+    </row>
+    <row r="1041" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1041" s="10"/>
+    </row>
+    <row r="1042" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1042" s="10"/>
+    </row>
+    <row r="1043" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1043" s="10"/>
+    </row>
+    <row r="1044" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1044" s="10"/>
+    </row>
+    <row r="1045" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1045" s="10"/>
+    </row>
+    <row r="1046" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1046" s="10"/>
+    </row>
+    <row r="1047" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1047" s="10"/>
+    </row>
+    <row r="1048" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1048" s="10"/>
+    </row>
+    <row r="1049" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1049" s="10"/>
+    </row>
+    <row r="1050" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1050" s="10"/>
+    </row>
+    <row r="1051" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1051" s="10"/>
+    </row>
+    <row r="1052" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1052" s="10"/>
+    </row>
+    <row r="1053" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1053" s="10"/>
+    </row>
+    <row r="1054" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1054" s="10"/>
+    </row>
+    <row r="1055" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1055" s="10"/>
+    </row>
+    <row r="1056" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1056" s="10"/>
+    </row>
+    <row r="1057" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1057" s="10"/>
+    </row>
+    <row r="1058" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1058" s="10"/>
+    </row>
+    <row r="1059" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I1059" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>